<commit_message>
Replace Quick Sketch with Doodle Stitch wall extensions
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.7</t>
+          <t>Alpha 0.1.8</t>
         </is>
       </c>
     </row>
@@ -647,12 +647,12 @@
     <row r="9" ht="88" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Quick Sketch status</t>
+          <t>Doodle Stitch status</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Flagged for review; its gameplay effect is unchanged.</t>
+          <t>Implemented replacement for Quick Sketch: endpoint connections with diminishing added HP.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Only Quick Sketch has been explicitly flagged by the player in this conversation; other candidates are hypotheses, not pick-rate data.</t>
+          <t>Quick Sketch was retired and replaced by Doodle Stitch following player feedback. Other review candidates are hypotheses, not pick-rate data.</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
     <row r="15" ht="88" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Quick Sketch</t>
+          <t>Doodle Stitch</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Your first stroke every wave is free.</t>
+          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; first valid stroke each wave only. Free strokes have no erasure/closure ink refund.</t>
+          <t>Endpoint snap reach 16px. New-length HP: 75%, 50%, 25%, then zero. Existing damage, oldest lifetime and summed group histories are preserved; erasing retains history.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -4510,7 +4510,7 @@
     <row r="15" ht="88" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Quick Sketch</t>
+          <t>Doodle Stitch</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -4520,22 +4520,22 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Your first stroke every wave is free.</t>
+          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>User flagged</t>
+          <t>Implemented replacement</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Rework candidate: try three discounted opening strokes, or an emergency free stroke earned by erasing. Compare against the value of one long free wall.</t>
+          <t>Replaces Quick Sketch. Playtest endpoint reach, the three diminishing HP additions, damaged-wall rescue and fourth-plus extensions without new HP.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
Make erasing wear paper, counter shots and trigger wall reactions
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -230,8 +230,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="MechanicsTable" displayName="MechanicsTable" ref="A1:C8" headerRowCount="1">
-  <autoFilter ref="A1:C8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="MechanicsTable" displayName="MechanicsTable" ref="A1:C10" headerRowCount="1">
+  <autoFilter ref="A1:C10"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Mechanic or specialization"/>
     <tableColumn id="2" name="Current behavior"/>
@@ -576,7 +576,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.8</t>
+          <t>Alpha 0.1.9</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3915,83 +3915,117 @@
     <row r="4" ht="88" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Closed shapes</t>
+          <t>Paper wear and tunnels</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>A stroke with more than six points and endpoints less than 22 pixels apart is a closed loop. Closed Loop/Fortress Geometry add durability and paid completion utility; related synergies add effects.</t>
+          <t>About 7 seconds of local active eraser rubbing tears a hole. Holes persist for the run, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>js/walls.js; js/upgrades.js</t>
+          <t>js/paper.js</t>
         </is>
       </c>
     </row>
     <row r="5" ht="88" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Stevie throws rocks</t>
+          <t>Erase combat</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Unlocked through rock upgrades or Pocket Pebbles. Automatically targets a nearby enemy within 210 pixels. Damage and rate grow with investment; Pocket Rocks also unlocks rock/ink synergies.</t>
+          <t>Erase small hostile pencils/spikes, sacrificing return damage. Erasing paid electric ink between surviving wall ends discharges up to 12 + 2 × Electric Ink level damage, limited to 0.8 × removed paid ink, with a 0.8-second wall cooldown retained by fragments. Erase Chonks’s windup support or Boingus’s fresh rebound support to stun for 1.4 seconds; each monster has a 6-second stumble cooldown.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>js/enemies.js; js/balance.js</t>
+          <t>js/paper.js; js/walls.js</t>
         </is>
       </c>
     </row>
     <row r="6" ht="88" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Specialization: Fortress</t>
+          <t>Closed shapes</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Defense-category upgrade weights ×3. Does not directly add wall HP.</t>
+          <t>A stroke with more than six points and endpoints less than 22 pixels apart is a closed loop. Closed Loop/Fortress Geometry add durability and paid completion utility; related synergies add effects.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>js/upgrades.js</t>
+          <t>js/walls.js; js/upgrades.js</t>
         </is>
       </c>
     </row>
     <row r="7" ht="88" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Specialization: Ink Alchemist</t>
+          <t>Stevie throws rocks</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Ink-category upgrade weights ×3. Does not directly add ink levels.</t>
+          <t>Unlocked through rock upgrades or Pocket Pebbles. Automatically targets a nearby enemy within 210 pixels. Damage and rate grow with investment; Pocket Rocks also unlocks rock/ink synergies.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>js/upgrades.js</t>
+          <t>js/enemies.js; js/balance.js</t>
         </is>
       </c>
     </row>
     <row r="8" ht="88" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Specialization: Fortress</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Defense-category upgrade weights ×3. Does not directly add wall HP.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="88" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Specialization: Ink Alchemist</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Ink-category upgrade weights ×3. Does not directly add ink levels.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="88" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Specialization: Chaos</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Adds +12 normal-reward rarity bonus; enemy HP scale ×1.08. No additional Legendary chances.</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>

</xml_diff>

<commit_message>
Limit paper shortcuts to chance encounters and animate early doodles
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.9</t>
+          <t>Alpha 0.1.10</t>
         </is>
       </c>
     </row>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>About 7 seconds of local active eraser rubbing tears a hole. Holes persist for the run, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
+          <t>About 7 seconds of local active eraser rubbing tears a hole. Holes persist for the run, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Give each drawing-tool rank distinct art and permanent wall durability
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -214,8 +214,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G11" headerRowCount="1">
-  <autoFilter ref="A1:G11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G10" headerRowCount="1">
+  <autoFilter ref="A1:G10"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Perk"/>
     <tableColumn id="2" name="Current ability"/>
@@ -576,7 +576,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.10</t>
+          <t>Alpha 0.1.11</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" ht="88" customHeight="1">
@@ -676,7 +676,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Quick Sketch was retired and replaced by Doodle Stitch following player feedback. Other review candidates are hypotheses, not pick-rate data.</t>
+          <t>Fresh Pencil was retired; legacy paid ranks receive a one-time scrap refund. Every Drawing Tool rank adds +8 base wall HP. Quick Sketch was retired and replaced by Doodle Stitch following player feedback. Other review candidates are hypotheses, not pick-rate data.</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Grow from Pencil to Mechanical Pencil (rank 3), Simple Pen (rank 6), and Scented Sharpie (rank 10). Pens unlock a third effect slot; Sharpies unlock a fourth.</t>
+          <t>Grow from Pencil to Mechanical Pencil (rank 3), Simple Pen (rank 6), and Scented Sharpie (rank 10). Every rank has its own artwork and adds +8 base wall HP. Pens unlock a third effect slot; Sharpies unlock a fourth.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -3544,12 +3544,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pencil · 2 effect slots</t>
+          <t>Pencil · 2 effect slots · +8 base wall HP</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Scented Sharpie · 4 effect slots</t>
+          <t>Scented Sharpie · 4 effect slots · +80 base wall HP</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -3666,12 +3666,12 @@
     <row r="7" ht="88" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Fresh Pencil</t>
+          <t>Lunchbox Band-Aids</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+8 starting wall HP per rank.</t>
+          <t>+8 starting/max Stevie HP per rank.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>+8 base wall HP</t>
+          <t>+8 Stevie HP</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>+32 base wall HP</t>
+          <t>+32 Stevie HP</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -3701,30 +3701,30 @@
     <row r="8" ht="88" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lunchbox Band-Aids</t>
+          <t>Pocket Pebbles</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+8 starting/max Stevie HP per rank.</t>
+          <t>Start throwing rocks: 3 damage per rank. Higher ranks throw a little faster.</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24, 40</t>
+          <t>5, 12, 24</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>+8 Stevie HP</t>
+          <t>3 starting rock damage · 1.5s between throws</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>+32 Stevie HP</t>
+          <t>9 starting rock damage · 1.3s between throws</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -3736,30 +3736,30 @@
     <row r="9" ht="88" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Pocket Pebbles</t>
+          <t>Lunch Money</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Start throwing rocks: 3 damage per rank. Higher ranks throw a little faster.</t>
+          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24</t>
+          <t>5, 12</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>3 starting rock damage · 1.5s between throws</t>
+          <t>+1 starting rerolls</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>9 starting rock damage · 1.3s between throws</t>
+          <t>+2 starting rerolls</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3771,68 +3771,33 @@
     <row r="10" ht="88" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lunch Money</t>
+          <t>Lucky Eraser</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+          <t>+2 starting Luck per rank, improving upgrade rarity odds.</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>5, 12</t>
+          <t>5, 12, 24, 40</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>+1 starting rerolls</t>
+          <t>+2 starting Luck</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>+2 starting rerolls</t>
+          <t>+8 starting Luck</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>js/notebook.js</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="88" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Lucky Eraser</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>+2 starting Luck per rank, improving upgrade rarity odds.</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>5, 12, 24, 40</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>+2 starting Luck</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>+8 starting Luck</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>js/notebook.js</t>
         </is>

</xml_diff>

<commit_message>
Add electric rock wall charges and bounded radial lightning bursts
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -183,8 +183,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I43" headerRowCount="1">
-  <autoFilter ref="A1:I43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I44" headerRowCount="1">
+  <autoFilter ref="A1:I44"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -242,8 +242,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J43" headerRowCount="1">
-  <autoFilter ref="A1:J43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J44" headerRowCount="1">
+  <autoFilter ref="A1:J44"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -576,7 +576,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.11</t>
+          <t>Alpha 0.1.13</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" ht="88" customHeight="1">
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1773,7 +1773,7 @@
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Pocket Rocks</t>
+          <t>Electric Rocks</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
+          <t>Unlock 4-damage rocks if needed. Rocks charge a short wall section for 2.4s, or burst sparks from Electric Ink walls. Sparks hit up to 8 nearby monsters for 4–9 damage. Each wall recovers for 1.1s. Max 6 levels.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1803,14 +1803,10 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Hot Rocks, Snowball Fight, Thunderstones</t>
-        </is>
-      </c>
+          <t>Max 6 levels. First wall crossed per rock; 2.4s charge within 48px of impact. Electric Ink burst reaches 103–118px, hits up to 8 surface monsters for 4–9 electric damage, and shares enemy electric recovery; 1.1s wall cooldown. Rocks keep flying. Thunderstones also enables this wall reaction.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1820,7 +1816,7 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Better Rocks</t>
+          <t>Pocket Rocks</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1830,7 +1826,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1853,7 +1849,11 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Hot Rocks, Snowball Fight, Thunderstones</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1863,7 +1863,7 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>Better Rocks</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1906,7 +1906,7 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Really Good Rocks</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Shared combat-healing budget: 6 HP/s.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1949,7 +1949,7 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Stevie Has Had Enough</t>
+          <t>Really Good Rocks</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1982,11 +1982,7 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Stevie the Unreasonable</t>
-        </is>
-      </c>
+      <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1996,40 +1992,44 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / rocks / survival</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Stevie the Unreasonable</t>
+        </is>
+      </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2039,7 +2039,7 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2049,27 +2049,27 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -2082,7 +2082,7 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2092,27 +2092,27 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
+          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -2125,7 +2125,7 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
+          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -2168,44 +2168,40 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Rocks, INFERNO</t>
-        </is>
-      </c>
+          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2215,7 +2211,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2225,7 +2221,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2250,7 +2246,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Ice Corridor, Snowball Fight, THE STORM, ABSOLUTE ZERO</t>
+          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Rocks, INFERNO</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2262,7 +2258,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2272,7 +2268,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2297,7 +2293,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
+          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Ice Corridor, Snowball Fight, THE STORM, ABSOLUTE ZERO</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2309,7 +2305,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2319,7 +2315,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2344,7 +2340,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO, ABSOLUTE ZERO</t>
+          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2356,7 +2352,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2366,7 +2362,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2391,7 +2387,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Power Lines, Thunderstones, THE STORM, TESLA CAGE</t>
+          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO, ABSOLUTE ZERO</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2403,7 +2399,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2413,7 +2409,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2438,7 +2434,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
+          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Power Lines, Thunderstones, THE STORM, TESLA CAGE</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2450,7 +2446,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2460,7 +2456,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2480,12 +2476,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2497,7 +2493,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2507,7 +2503,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2527,12 +2523,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
+          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2544,7 +2540,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2554,7 +2550,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2579,7 +2575,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Event Horizon, THE BLACK HOLE</t>
+          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2591,7 +2587,7 @@
     <row r="42" ht="88" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2601,7 +2597,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2624,7 +2620,11 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Event Horizon, THE BLACK HOLE</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2634,7 +2634,7 @@
     <row r="43" ht="88" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Death Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2664,11 +2664,54 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
       <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="88" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Death Ink</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>
@@ -3244,7 +3287,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Stevie's rocks can chain lightning.</t>
+          <t>Stevie's rocks chain lightning and burst sparks from Electric Ink walls.</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4809,7 +4852,7 @@
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Pocket Rocks</t>
+          <t>Electric Rocks</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -4819,7 +4862,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
+          <t>Unlock 4-damage rocks if needed. Rocks charge a short wall section for 2.4s, or burst sparks from Electric Ink walls. Sparks hit up to 8 nearby monsters for 4–9 damage. Each wall recovers for 1.1s. Max 6 levels.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4841,7 +4884,7 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Better Rocks</t>
+          <t>Pocket Rocks</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -4851,7 +4894,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -4873,7 +4916,7 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>Better Rocks</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -4883,7 +4926,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -4905,7 +4948,7 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Really Good Rocks</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -4915,7 +4958,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -4937,7 +4980,7 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Stevie Has Had Enough</t>
+          <t>Really Good Rocks</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -4947,7 +4990,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -4969,17 +5012,17 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / rocks / survival</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -5001,7 +5044,7 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -5011,7 +5054,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -5033,7 +5076,7 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -5043,24 +5086,20 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr"/>
@@ -5069,7 +5108,7 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -5079,20 +5118,24 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
+        </is>
+      </c>
       <c r="G32" s="4" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr"/>
@@ -5101,17 +5144,17 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -5133,7 +5176,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -5143,7 +5186,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5165,7 +5208,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -5175,7 +5218,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -5197,7 +5240,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -5207,7 +5250,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -5229,7 +5272,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -5239,7 +5282,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -5261,7 +5304,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -5271,7 +5314,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -5293,7 +5336,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -5303,7 +5346,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -5325,7 +5368,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -5335,24 +5378,20 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="4" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr"/>
@@ -5361,7 +5400,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -5371,20 +5410,24 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
+        </is>
+      </c>
       <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr"/>
@@ -5393,7 +5436,7 @@
     <row r="42" ht="88" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -5403,7 +5446,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -5425,7 +5468,7 @@
     <row r="43" ht="88" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Death Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -5435,7 +5478,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -5454,13 +5497,45 @@
       <c r="I43" s="4" t="inlineStr"/>
       <c r="J43" s="4" t="inlineStr"/>
     </row>
+    <row r="44" ht="88" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Death Ink</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Not rated</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
+    <dataValidation sqref="G2:G44" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Keep,Rework,Remove,Test first"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Unlock run-only Doodle Scrap discoveries and five paper-ball elements
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -183,8 +183,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I44" headerRowCount="1">
-  <autoFilter ref="A1:I44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I43" headerRowCount="1">
+  <autoFilter ref="A1:I43"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -214,8 +214,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G10" headerRowCount="1">
-  <autoFilter ref="A1:G10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G11" headerRowCount="1">
+  <autoFilter ref="A1:G11"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Perk"/>
     <tableColumn id="2" name="Current ability"/>
@@ -230,8 +230,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="MechanicsTable" displayName="MechanicsTable" ref="A1:C10" headerRowCount="1">
-  <autoFilter ref="A1:C10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="MechanicsTable" displayName="MechanicsTable" ref="A1:C11" headerRowCount="1">
+  <autoFilter ref="A1:C11"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Mechanic or specialization"/>
     <tableColumn id="2" name="Current behavior"/>
@@ -242,8 +242,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J44" headerRowCount="1">
-  <autoFilter ref="A1:J44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J43" headerRowCount="1">
+  <autoFilter ref="A1:J43"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" ht="88" customHeight="1">
@@ -607,7 +607,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" ht="88" customHeight="1">
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1773,7 +1773,7 @@
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Electric Rocks</t>
+          <t>Pocket Rocks</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Unlock 4-damage rocks if needed. Rocks charge a short wall section for 2.4s, or burst sparks from Electric Ink walls. Sparks hit up to 8 nearby monsters for 4–9 damage. Each wall recovers for 1.1s. Max 6 levels.</t>
+          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1803,10 +1803,14 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Max 6 levels. First wall crossed per rock; 2.4s charge within 48px of impact. Electric Ink burst reaches 103–118px, hits up to 8 surface monsters for 4–9 electric damage, and shares enemy electric recovery; 1.1s wall cooldown. Rocks keep flying. Thunderstones also enables this wall reaction.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Hot Rocks, Snowball Fight, Thunderstones</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1816,7 +1820,7 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Pocket Rocks</t>
+          <t>Better Rocks</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1826,7 +1830,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
+          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1849,11 +1853,7 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Hot Rocks, Snowball Fight, Thunderstones</t>
-        </is>
-      </c>
+      <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1863,7 +1863,7 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Better Rocks</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Shared combat-healing budget: 6 HP/s.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1906,7 +1906,7 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>Really Good Rocks</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1949,7 +1949,7 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Really Good Rocks</t>
+          <t>Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1982,7 +1982,11 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Stevie the Unreasonable</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1992,44 +1996,40 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Stevie Has Had Enough</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Stevie the Unreasonable</t>
-        </is>
-      </c>
+          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2039,7 +2039,7 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2049,27 +2049,27 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -2082,7 +2082,7 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2092,27 +2092,27 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -2125,7 +2125,7 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
+          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -2168,40 +2168,44 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Ink effects</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Rocks, INFERNO</t>
+        </is>
+      </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2211,7 +2215,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2221,7 +2225,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2246,7 +2250,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Rocks, INFERNO</t>
+          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Ice Corridor, Snowball Fight, THE STORM, ABSOLUTE ZERO</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2258,7 +2262,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2268,7 +2272,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2293,7 +2297,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Ice Corridor, Snowball Fight, THE STORM, ABSOLUTE ZERO</t>
+          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2305,7 +2309,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2315,7 +2319,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2340,7 +2344,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
+          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO, ABSOLUTE ZERO</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2352,7 +2356,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2362,7 +2366,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2387,7 +2391,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO, ABSOLUTE ZERO</t>
+          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Power Lines, Thunderstones, THE STORM, TESLA CAGE</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2399,7 +2403,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2409,7 +2413,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2434,7 +2438,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Power Lines, Thunderstones, THE STORM, TESLA CAGE</t>
+          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2446,7 +2450,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2456,7 +2460,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2476,12 +2480,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
+          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2493,7 +2497,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2503,7 +2507,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2523,12 +2527,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2540,7 +2544,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2550,7 +2554,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2575,7 +2579,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
+          <t>Event Horizon, THE BLACK HOLE</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2587,7 +2591,7 @@
     <row r="42" ht="88" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2597,7 +2601,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2620,11 +2624,7 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>Event Horizon, THE BLACK HOLE</t>
-        </is>
-      </c>
+      <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2634,7 +2634,7 @@
     <row r="43" ht="88" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Death Ink</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2664,54 +2664,11 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
       <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>js/upgrades.js</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="88" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Death Ink</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Ink effects</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>
@@ -3482,7 +3439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3569,30 +3526,30 @@
     <row r="3" ht="88" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Your Drawing Tool</t>
+          <t>Doodle Scraps</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Grow from Pencil to Mechanical Pencil (rank 3), Simple Pen (rank 6), and Scented Sharpie (rank 10). Every rank has its own artwork and adds +8 base wall HP. Pens unlock a third effect slot; Sharpies unlock a fourth.</t>
+          <t>Unlock mysterious paper drops in future runs, from any wave. Draw through one and choose a temporary element for Stevie’s paper balls. Finds last only for that run.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>5, 8, 12, 16, 20, 24, 30, 36, 44, 55</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pencil · 2 effect slots · +8 base wall HP</t>
+          <t>Doodle Scraps can drop from wave 1</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Scented Sharpie · 4 effect slots · +80 base wall HP</t>
+          <t>Doodle Scraps can drop from wave 1</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -3604,30 +3561,30 @@
     <row r="4" ht="88" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Bigger Starting Tank</t>
+          <t>Your Drawing Tool</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>+20 starting/max ink per rank.</t>
+          <t>Grow from Pencil to Mechanical Pencil (rank 3), Simple Pen (rank 6), and Scented Sharpie (rank 10). Every rank has its own artwork and adds +8 base wall HP. Pens unlock a third effect slot; Sharpies unlock a fourth.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24, 40, 60</t>
+          <t>5, 8, 12, 16, 20, 24, 30, 36, 44, 55</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>+20 starting/max ink</t>
+          <t>Pencil · 2 effect slots · +8 base wall HP</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>+100 starting/max ink</t>
+          <t>Scented Sharpie · 4 effect slots · +80 base wall HP</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -3639,30 +3596,30 @@
     <row r="5" ht="88" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Refill Practice</t>
+          <t>Bigger Starting Tank</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+1 starting ink regeneration per second per rank. Stacks with run upgrades.</t>
+          <t>+20 starting/max ink per rank.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24</t>
+          <t>5, 12, 24, 40, 60</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>+1 starting ink/s</t>
+          <t>+20 starting/max ink</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>+3 starting ink/s</t>
+          <t>+100 starting/max ink</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3674,30 +3631,30 @@
     <row r="6" ht="88" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Extra Credit</t>
+          <t>Refill Practice</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Start every run with four reward choices instead of three. Boss rewards already have four.</t>
+          <t>+1 starting ink regeneration per second per rank. Stacks with run upgrades.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>5, 12, 24</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>4 reward choices from the first wave</t>
+          <t>+1 starting ink/s</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>4 reward choices from the first wave</t>
+          <t>+3 starting ink/s</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -3709,30 +3666,30 @@
     <row r="7" ht="88" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Lunchbox Band-Aids</t>
+          <t>Extra Credit</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+8 starting/max Stevie HP per rank.</t>
+          <t>Start every run with four reward choices instead of three. Boss rewards already have four.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24, 40</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>+8 Stevie HP</t>
+          <t>4 reward choices from the first wave</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>+32 Stevie HP</t>
+          <t>4 reward choices from the first wave</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -3744,30 +3701,30 @@
     <row r="8" ht="88" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Pocket Pebbles</t>
+          <t>Lunchbox Band-Aids</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Start throwing rocks: 3 damage per rank. Higher ranks throw a little faster.</t>
+          <t>+8 starting/max Stevie HP per rank.</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24</t>
+          <t>5, 12, 24, 40</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>3 starting rock damage · 1.5s between throws</t>
+          <t>+8 Stevie HP</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>9 starting rock damage · 1.3s between throws</t>
+          <t>+32 Stevie HP</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -3779,30 +3736,30 @@
     <row r="9" ht="88" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Lunch Money</t>
+          <t>Paper Ball Practice</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+          <t>Start throwing crumpled paper: 3 damage per rank. Higher ranks throw a little faster.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>5, 12</t>
+          <t>5, 12, 24</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>+1 starting rerolls</t>
+          <t>3 starting paper-ball damage · 1.5s between throws</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>+2 starting rerolls</t>
+          <t>9 starting paper-ball damage · 1.3s between throws</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3814,33 +3771,68 @@
     <row r="10" ht="88" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Lunch Money</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>5, 12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting rerolls</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>+2 starting rerolls</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>js/notebook.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="88" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Lucky Eraser</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>+2 starting Luck per rank, improving upgrade rarity odds.</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>5, 12, 24, 40</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>+2 starting Luck</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>+8 starting Luck</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>js/notebook.js</t>
         </is>
@@ -3861,7 +3853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3974,12 +3966,12 @@
     <row r="7" ht="88" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Stevie throws rocks</t>
+          <t>Stevie throws paper balls</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Unlocked through rock upgrades or Pocket Pebbles. Automatically targets a nearby enemy within 210 pixels. Damage and rate grow with investment; Pocket Rocks also unlocks rock/ink synergies.</t>
+          <t>Unlocked through throwing upgrades, Paper Ball Practice or a Doodle Scrap discovery. Automatically targets a nearby enemy within 210 pixels. Damage and rate grow with investment; Pocket Rocks also unlocks rock/ink synergies.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -3991,29 +3983,29 @@
     <row r="8" ht="88" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Specialization: Fortress</t>
+          <t>Doodle Scraps</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Defense-category upgrade weights ×3. Does not directly add wall HP.</t>
+          <t>Permanent Notebook unlock costs 25 saved scraps. From wave 1, eligible normal kills have an 8% drop chance; first drop guaranteed by eight eligible kills. Minimum 20 combat seconds between drops, one ground pickup at a time, max four per run; drops last 45 combat seconds. Finish a drawing through a pickup to reel it in and pause for two random elements. Fire, electric, poison, frost and eraser paper replace the current element and last only for the run; no wave-reward or ink slots used. Choosing an element unlocks 4-damage, 1.6s throws if needed. Bosses/helpers and development tests do not drop discoveries.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>js/upgrades.js</t>
+          <t>js/doodle-scraps.js; js/notebook.js</t>
         </is>
       </c>
     </row>
     <row r="9" ht="88" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Specialization: Ink Alchemist</t>
+          <t>Specialization: Fortress</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ink-category upgrade weights ×3. Does not directly add ink levels.</t>
+          <t>Defense-category upgrade weights ×3. Does not directly add wall HP.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -4025,15 +4017,32 @@
     <row r="10" ht="88" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Specialization: Ink Alchemist</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Ink-category upgrade weights ×3. Does not directly add ink levels.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="88" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Specialization: Chaos</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Adds +12 normal-reward rarity bonus; enemy HP scale ×1.08. No additional Legendary chances.</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>
@@ -4054,7 +4063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4852,7 +4861,7 @@
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Electric Rocks</t>
+          <t>Pocket Rocks</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -4862,7 +4871,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Unlock 4-damage rocks if needed. Rocks charge a short wall section for 2.4s, or burst sparks from Electric Ink walls. Sparks hit up to 8 nearby monsters for 4–9 damage. Each wall recovers for 1.1s. Max 6 levels.</t>
+          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -4884,7 +4893,7 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Pocket Rocks</t>
+          <t>Better Rocks</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -4894,7 +4903,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
+          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -4916,7 +4925,7 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Better Rocks</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -4926,7 +4935,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -4948,7 +4957,7 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>Really Good Rocks</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -4958,7 +4967,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -4980,7 +4989,7 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Really Good Rocks</t>
+          <t>Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -4990,7 +4999,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -5012,17 +5021,17 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Stevie Has Had Enough</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -5044,7 +5053,7 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -5054,7 +5063,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -5076,7 +5085,7 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -5086,20 +5095,24 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
+        </is>
+      </c>
       <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr"/>
@@ -5108,7 +5121,7 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -5118,24 +5131,20 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="4" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr"/>
@@ -5144,17 +5153,17 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Ink effects</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -5176,7 +5185,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -5186,7 +5195,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5208,7 +5217,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -5218,7 +5227,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -5240,7 +5249,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -5250,7 +5259,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -5272,7 +5281,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -5282,7 +5291,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -5304,7 +5313,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -5314,7 +5323,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -5336,7 +5345,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -5346,7 +5355,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -5368,7 +5377,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -5378,20 +5387,24 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
+        </is>
+      </c>
       <c r="G40" s="4" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr"/>
@@ -5400,7 +5413,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -5410,24 +5423,20 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr"/>
@@ -5436,7 +5445,7 @@
     <row r="42" ht="88" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -5446,7 +5455,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -5468,7 +5477,7 @@
     <row r="43" ht="88" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Death Ink</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -5478,7 +5487,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -5497,45 +5506,13 @@
       <c r="I43" s="4" t="inlineStr"/>
       <c r="J43" s="4" t="inlineStr"/>
     </row>
-    <row r="44" ht="88" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Death Ink</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Ink effects</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Not rated</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="4" t="inlineStr"/>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="4" t="inlineStr"/>
-      <c r="J44" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G44" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
+    <dataValidation sqref="G2:G43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Keep,Rework,Remove,Test first"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Require three eraser passes for Ruff and refresh paper each wave
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.13</t>
+          <t>Alpha 0.1.15</t>
         </is>
       </c>
     </row>
@@ -3920,7 +3920,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>About 7 seconds of local active eraser rubbing tears a hole. Holes persist for the run, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
+          <t>About 2.5 seconds of local active eraser rubbing tears a hole. Each wave starts with fresh paper; wear and holes reset, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Stack illustrated Doodle Scraps with drawing tricks and desktop throw aiming
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -11,16 +11,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Upgrades" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synergies" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notebook Perks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retuning Review" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doodle Scraps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mechanics" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retuning Review" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Read Me'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Run Upgrades'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Synergies'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Notebook Perks'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Mechanics'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Retuning Review'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Doodle Scraps'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Mechanics'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Retuning Review'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -230,7 +232,20 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="MechanicsTable" displayName="MechanicsTable" ref="A1:C11" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DoodleScrapsTable" displayName="DoodleScrapsTable" ref="A1:D15" headerRowCount="1">
+  <autoFilter ref="A1:D15"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Note"/>
+    <tableColumn id="2" name="Rarity"/>
+    <tableColumn id="3" name="Current effect"/>
+    <tableColumn id="4" name="Source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="MechanicsTable" displayName="MechanicsTable" ref="A1:C11" headerRowCount="1">
   <autoFilter ref="A1:C11"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Mechanic or specialization"/>
@@ -241,8 +256,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J43" headerRowCount="1">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J43" headerRowCount="1">
   <autoFilter ref="A1:J43"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Upgrade"/>
@@ -576,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.16</t>
+          <t>Alpha 0.1.18</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3546,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Unlock mysterious paper drops in future runs, from any wave. Draw through one and choose a temporary element for Stevie’s paper balls. Finds last only for that run.</t>
+          <t>Unlock mysterious paper drops in future runs, from any wave. Draw through one and choose a stacking trick for Stevie’s paper balls. Discover elemental throws, wall rides, decoys and Connect the Dots. Finds last only for that run.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -3853,6 +3868,360 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="105" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Rarity</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Current effect</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="88" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Hot Off the Page</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ignite enemies. More copies strengthen the burn.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="88" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Static Scribble</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Spark enemies and charge crossed walls.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="88" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Questionable Lunch</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Add stacking poison. Stevie insists it is still good.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="88" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Cold Shoulder</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Briefly chill enemies. Repeat copies improve the chill, with a control cap.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="88" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Correction Notice</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Add eraser damage. Each hit wipes one chunk off Ruff.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="88" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Long Distance Learning</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Reach farther enemies. Repeat copies extend range with diminishing returns.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="88" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Second Draft</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Every few throws, send a second ball at a different enemy. Copies make this happen more often.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="88" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Follow the Underline</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Paper balls ride your lines, then launch from the far end with extra range.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="88" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Static Cling</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Repeated electric hits prime an enemy to stick briefly to the next wall. Includes a basic electric effect if needed.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="88" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Ash Impostor</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Hit a burning enemy to shed a smoky decoy that distracts nearby monsters. Includes basic fire if needed.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="88" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Bubble Trouble</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Repeated poison hits inflate a wandering bubble. Erase it to pop and stagger the monster. Includes basic poison if needed.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="88" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Cross Out</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Erasing hostile pencils or spikes turns their remains into friendly paper throws.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="88" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Connect the Dots</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Paper hits mark monsters with bright dots. Draw through two dots to snap a colorful tether between them!</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="88" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Bad Influence</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Ash decoys carry your paper elements. Monsters biting one receive those effects. Includes Ash Impostor if needed.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3971,7 +4340,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Unlocked through throwing upgrades, Paper Ball Practice or a Doodle Scrap discovery. Automatically targets a nearby enemy within 210 pixels. Damage and rate grow with investment; Pocket Rocks also unlocks rock/ink synergies.</t>
+          <t>Unlocked through throwing upgrades, Paper Ball Practice or a Doodle Scrap discovery. Automatically targets a nearby enemy within 210 pixels before range notes. Desktop WASD steers throws while held; releasing restores auto-aim. Touch keeps auto-aim. Damage and rate grow with investment; Pocket Rocks also unlocks rock/ink synergies.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -3988,12 +4357,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Permanent Notebook unlock costs 25 saved scraps. From wave 1, eligible normal kills have an 8% drop chance; first drop guaranteed by eight eligible kills. Minimum 20 combat seconds between drops, one ground pickup at a time, max four per run; drops last 45 combat seconds. Finish a drawing through a pickup to reel it in and pause for two random elements. Fire, electric, poison, frost and eraser paper replace the current element and last only for the run; no wave-reward or ink slots used. Choosing an element unlocks 4-damage, 1.6s throws if needed. Bosses/helpers and development tests do not drop discoveries.</t>
+          <t>Permanent Notebook unlock costs 25 saved scraps. Wave budgets: 25% zero, 40% one, 25% two, 10% three; eligible normal kills reveal the budget, with 10 combat seconds between discoveries. One pickup at a time, lasts 45 seconds. Draw through it to pause and choose one of two distinct notes of the same rarity. Tier odds: Common 55%, Uncommon 28%, Rare 13%, Epic 4%. No Legendary notes yet. All notes and duplicate copies stack for the run, with bounded control/procs and diminishing range. New notes do not change throws already in flight. No wave-reward slots used; development tests and boss/helpers excluded.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/notebook.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/notebook.js</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4426,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add stackable legendary paper-ball notes and split throws
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -232,8 +232,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DoodleScrapsTable" displayName="DoodleScrapsTable" ref="A1:D15" headerRowCount="1">
-  <autoFilter ref="A1:D15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DoodleScrapsTable" displayName="DoodleScrapsTable" ref="A1:D22" headerRowCount="1">
+  <autoFilter ref="A1:D22"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Note"/>
     <tableColumn id="2" name="Rarity"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.18</t>
+          <t>Alpha 0.1.19</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4005,7 +4005,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4088,12 +4088,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Repeated electric hits prime an enemy to stick briefly to the next wall. Includes a basic electric effect if needed.</t>
+          <t>Repeated electric hits make nearby monsters cling to each other in slow, sparking clumps. Includes basic electricity.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4137,7 +4137,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,161 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>js/doodle-scraps.js; js/doodle-tricks.js</t>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="88" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Split Decision</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>On its first hit, a ball splits toward two different nearby enemies. Each copy adds one generation. Children carry your notes and retain 50% damage, improving slightly with copies.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="88" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Rapid Scribble</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Throw paper balls 5% faster per copy. Additive speed bonuses have no rank cap.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="88" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Round Trip</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Paper balls orbit struck monsters and repeatedly deal their paper damage until that monster dies. Split children can orbit too; laps never split again.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="88" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Extra Credit</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Every hit hops to another enemy within 90px and adds +1 physical damage per copy. No hop limit. If nobody is nearby, the ball waits for its next short hop.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="88" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Wallflowers</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Finished throws perch on nearby walls, then launch again when monsters approach. The balls keep your notes and can be reused while their wall survives.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="88" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Carbon Copy</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Cross any wall to fire two straight paper duplicates out its sides. They deal double physical damage and carry your notes. Each ball copies once per wall; duplicates cannot make more carbon copies.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="88" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Extra Ink</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Black paper balls splash ink on impact: fully heal nearby walls, extend both ends of open walls, and refill 5 ink per copy on hit. Free growth does not create paid ink to reclaim.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>js/doodle-scraps.js; js/doodle-tricks.js; js/paper-tricks.js</t>
         </is>
       </c>
     </row>
@@ -4357,7 +4511,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Permanent Notebook unlock costs 25 saved scraps. Wave budgets: 25% zero, 40% one, 25% two, 10% three; eligible normal kills reveal the budget, with 10 combat seconds between discoveries. One pickup at a time, lasts 45 seconds. Draw through it to pause and choose one of two distinct notes of the same rarity. Tier odds: Common 55%, Uncommon 28%, Rare 13%, Epic 4%. No Legendary notes yet. All notes and duplicate copies stack for the run, with bounded control/procs and diminishing range. New notes do not change throws already in flight. No wave-reward slots used; development tests and boss/helpers excluded.</t>
+          <t>Permanent Notebook unlock costs 25 saved scraps. Wave budgets: 25% zero, 40% one, 25% two, 10% three; eligible normal kills reveal the budget, with 10 combat seconds between discoveries. One pickup at a time, lasts 45 seconds. Draw through it to pause and choose one of two distinct notes of the same rarity. Tier odds: Common 55%, Uncommon 28%, Rare 13%, Epic 3.7%, Legendary 0.3% per discovery. Five Legendary paper-ball behaviors are available. All notes and duplicate copies stack for the run, with bounded control/procs and diminishing range. New notes do not change throws already in flight. No wave-reward slots used; development tests and boss/helpers excluded.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Give early enemies distinct threats and fix paper wear
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.19</t>
+          <t>Alpha 0.1.20</t>
         </is>
       </c>
     </row>
@@ -4443,7 +4443,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>About 2.5 seconds of local active eraser rubbing tears a hole. Each wave starts with fresh paper; wear and holes reset, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
+          <t>About 2 seconds of local active eraser rubbing tears a hole. Each wave starts with fresh paper; wear and holes reset, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -4460,7 +4460,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Erase small hostile pencils/spikes, sacrificing return damage. Erasing paid electric ink between surviving wall ends discharges up to 12 + 2 × Electric Ink level damage, limited to 0.8 × removed paid ink, with a 0.8-second wall cooldown retained by fragments. Erase Chonks’s windup support or Boingus’s fresh rebound support to stun for 1.4 seconds; each monster has a 6-second stumble cooldown.</t>
+          <t>Erase small hostile pencils/spikes, sacrificing return damage. Erasing paid electric ink between surviving wall ends discharges up to 12 + 2 × Electric Ink level damage, limited to 0.8 × removed paid ink, with a 0.8-second wall cooldown retained by fragments. Erase Chonks’s recovery support or Boingus’s fresh rebound support to stun for 1.4 seconds; each monster has a 6-second stumble cooldown.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Retire duplicate walls and reduce elemental wall clutter
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -185,8 +185,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I43" headerRowCount="1">
-  <autoFilter ref="A1:I43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I41" headerRowCount="1">
+  <autoFilter ref="A1:I41"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -203,8 +203,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SynergiesTable" displayName="SynergiesTable" ref="A1:D33" headerRowCount="1">
-  <autoFilter ref="A1:D33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SynergiesTable" displayName="SynergiesTable" ref="A1:D30" headerRowCount="1">
+  <autoFilter ref="A1:D30"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Synergy"/>
     <tableColumn id="2" name="Kind"/>
@@ -257,8 +257,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J43" headerRowCount="1">
-  <autoFilter ref="A1:J43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J41" headerRowCount="1">
+  <autoFilter ref="A1:J41"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.20</t>
+          <t>Alpha 0.1.22</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" ht="88" customHeight="1">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" ht="88" customHeight="1">
@@ -691,7 +691,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Fresh Pencil was retired; legacy paid ranks receive a one-time scrap refund. Every Drawing Tool rank adds +8 base wall HP. Quick Sketch was retired and replaced by Doodle Stitch following player feedback. Other review candidates are hypotheses, not pick-rate data.</t>
+          <t>Fresh Pencil was retired; legacy paid ranks receive a one-time scrap refund. Every Drawing Tool rank adds +8 base wall HP. Quick Sketch was retired and replaced by Doodle Stitch following player feedback. Double Stroke, Triple Stroke and their parallel-wall synergies were retired to reduce clutter; one stroke creates one wall. Other review candidates are hypotheses, not pick-rate data.</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1346,7 +1346,7 @@
     <row r="14" ht="88" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Double Stroke</t>
+          <t>Doodle Stitch</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Each stroke adds a parallel wall with 60% of the original durability.</t>
+          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1376,14 +1376,10 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; disabled when parallel walls are already unlocked.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Ice Corridor, ABSOLUTE ZERO</t>
-        </is>
-      </c>
+          <t>Endpoint snap reach 16px. New-length HP: 75%, 50%, 25%, then zero. Existing damage, oldest lifetime and summed group histories are preserved; erasing retains history.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1393,37 +1389,37 @@
     <row r="15" ht="88" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Doodle Stitch</t>
+          <t>Patch Job</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
+          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Endpoint snap reach 16px. New-length HP: 75%, 50%, 25%, then zero. Existing damage, oldest lifetime and summed group histories are preserved; erasing retains history.</t>
+          <t>Shared repair-on-kill budget: 12 wall HP/s across all walls.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -1436,17 +1432,17 @@
     <row r="16" ht="88" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Patch Job</t>
+          <t>Freehand</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
+          <t>Spend 80 real ink to charge a limited free-ink bank. Stacking increases the free bank.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1466,7 +1462,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Shared repair-on-kill budget: 12 wall HP/s across all walls.</t>
+          <t>Charges from real paid ink, not free strokes/copies; threshold 80; initial bank 40, +20 per extra level.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1479,7 +1475,7 @@
     <row r="17" ht="88" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Freehand</t>
+          <t>Living Fountain Pen</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1489,7 +1485,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Spend 80 real ink to charge a limited free-ink bank. Stacking increases the free bank.</t>
+          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1509,7 +1505,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Charges from real paid ink, not free strokes/copies; threshold 80; initial bank 40, +20 per extra level.</t>
+          <t>Repeat level n multiplies regeneration by 1 + 0.35 / (1 + 0.5 × (n−1)).</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1522,7 +1518,7 @@
     <row r="18" ht="88" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Living Fountain Pen</t>
+          <t>Bottomless Pen</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1532,7 +1528,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
+          <t>Per level: +40 max ink and +2 ink/s at first, with smaller regeneration bonuses on repeats.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1552,7 +1548,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Repeat level n multiplies regeneration by 1 + 0.35 / (1 + 0.5 × (n−1)).</t>
+          <t>Each level adds 40 max ink; regeneration repeats use 2 / (1 + 0.4 × (n−1)).</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -1565,44 +1561,40 @@
     <row r="19" ht="88" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Triple Stroke</t>
+          <t>Fortress Geometry</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Every stroke adds TWO parallel walls, each with 60% durability.</t>
+          <t>Per level: +50% closed-shape durability. Shares Closed Loop’s diminishing ink refund, completion repair and enclosed-enemy damage bonus (15% / 15% / 10% at the first utility level).</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>legendary</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Legendary-only, one-time unlock; two copies replace the single Double Stroke copy.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Ice Corridor, Power Lines, ABSOLUTE ZERO</t>
-        </is>
-      </c>
+          <t>Shares diminishing loop utility with Closed Loop; free strokes/copies do not earn ink refunds.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1612,17 +1604,17 @@
     <row r="20" ht="88" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Bottomless Pen</t>
+          <t>Bandages</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Stevie / rocks / survival</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Per level: +40 max ink and +2 ink/s at first, with smaller regeneration bonuses on repeats.</t>
+          <t>Heal 8 extra HP between waves.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1642,7 +1634,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Each level adds 40 max ink; regeneration repeats use 2 / (1 + 0.4 × (n−1)).</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1655,17 +1647,17 @@
     <row r="21" ht="88" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Fortress Geometry</t>
+          <t>Helmet</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Stevie / rocks / survival</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Per level: +50% closed-shape durability. Shares Closed Loop’s diminishing ink refund, completion repair and enclosed-enemy damage bonus (15% / 15% / 10% at the first utility level).</t>
+          <t>Stevie takes 10% less contact damage.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1685,10 +1677,14 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Shares diminishing loop utility with Closed Loop; free strokes/copies do not earn ink refunds.</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>Damage reduction capped at 55%; awarded levels respect remaining cap.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Human Pinball</t>
+        </is>
+      </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1698,7 +1694,7 @@
     <row r="22" ht="88" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Bandages</t>
+          <t>Pocket Rocks</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1708,7 +1704,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Heal 8 extra HP between waves.</t>
+          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1731,7 +1727,11 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Hot Rocks, Snowball Fight, Thunderstones</t>
+        </is>
+      </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1741,7 +1741,7 @@
     <row r="23" ht="88" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Helmet</t>
+          <t>Better Rocks</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Stevie takes 10% less contact damage.</t>
+          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1771,14 +1771,10 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Damage reduction capped at 55%; awarded levels respect remaining cap.</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Human Pinball</t>
-        </is>
-      </c>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1788,7 +1784,7 @@
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Pocket Rocks</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1798,7 +1794,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
+          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1818,14 +1814,10 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Hot Rocks, Snowball Fight, Thunderstones</t>
-        </is>
-      </c>
+          <t>Shared combat-healing budget: 6 HP/s.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1835,7 +1827,7 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Better Rocks</t>
+          <t>Really Good Rocks</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1845,7 +1837,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1878,7 +1870,7 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1888,7 +1880,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1908,10 +1900,14 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s.</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Stevie the Unreasonable</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1921,37 +1917,37 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Really Good Rocks</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1964,17 +1960,17 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Stevie Has Had Enough</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1994,14 +1990,10 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Stevie the Unreasonable</t>
-        </is>
-      </c>
+          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2011,7 +2003,7 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2021,7 +2013,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2041,7 +2033,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -2054,7 +2046,7 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2064,27 +2056,27 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -2097,40 +2089,44 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Ink effects</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Rocks, INFERNO</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2140,40 +2136,44 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Ink effects</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2183,7 +2183,7 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Rocks, INFERNO</t>
+          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2230,7 +2230,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Ice Corridor, Snowball Fight, THE STORM, ABSOLUTE ZERO</t>
+          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2277,7 +2277,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
+          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunderstones, THE STORM, TESLA CAGE</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2324,7 +2324,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO, ABSOLUTE ZERO</t>
+          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2371,7 +2371,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2401,12 +2401,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Power Lines, Thunderstones, THE STORM, TESLA CAGE</t>
+          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2418,7 +2418,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
+          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2465,7 +2465,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2495,12 +2495,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+          <t>Event Horizon, THE BLACK HOLE</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2512,7 +2512,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2545,11 +2545,7 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
-        </is>
-      </c>
+      <c r="H40" s="2" t="inlineStr"/>
       <c r="I40" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2559,7 +2555,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Death Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2569,7 +2565,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2589,101 +2585,11 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>Event Horizon, THE BLACK HOLE</t>
-        </is>
-      </c>
+          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
       <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>js/upgrades.js</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="88" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Chaos Ink</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Ink effects</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>js/upgrades.js</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="88" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Death Ink</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Ink effects</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>
@@ -2704,7 +2610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3090,7 +2996,7 @@
     <row r="18" ht="88" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Ice Corridor</t>
+          <t>Blood Patch</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -3100,19 +3006,19 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink, Double Stroke (or Triple Stroke)</t>
+          <t>Vampire Ink, Patchwork</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>The space between parallel walls chills nearby enemies.</t>
+          <t>Repairing walls also heals Stevie.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="88" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Power Lines</t>
+          <t>Needlepoint</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -3122,19 +3028,19 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink, Triple Stroke</t>
+          <t>Poison Ink, Fine Tip</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Triple walls pulse electricity into enemies caught nearby.</t>
+          <t>Cheap thin lines stack poison much faster.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="88" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Blood Patch</t>
+          <t>Heavy Artillery</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -3144,19 +3050,19 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink, Patchwork</t>
+          <t>Blast Ink, Fat Marker</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Repairing walls also heals Stevie.</t>
+          <t>Thicker walls create larger explosions.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="88" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Needlepoint</t>
+          <t>Hot Rocks</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -3166,19 +3072,19 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink, Fine Tip</t>
+          <t>Fire Ink, Pocket Rocks</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Cheap thin lines stack poison much faster.</t>
+          <t>Stevie's rocks ignite enemies.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="88" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Heavy Artillery</t>
+          <t>Snowball Fight</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -3188,19 +3094,19 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink, Fat Marker</t>
+          <t>Frost Ink, Pocket Rocks</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Thicker walls create larger explosions.</t>
+          <t>Stevie's rocks chill and sometimes freeze enemies.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="88" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Hot Rocks</t>
+          <t>Thunderstones</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -3210,19 +3116,19 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink, Pocket Rocks</t>
+          <t>Electric Ink, Pocket Rocks</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Stevie's rocks ignite enemies.</t>
+          <t>Stevie's rocks chain lightning and burst sparks from Electric Ink walls.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Snowball Fight</t>
+          <t>Stevie the Unreasonable</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -3232,19 +3138,19 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink, Pocket Rocks</t>
+          <t>Vampire Ink, Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Stevie's rocks chill and sometimes freeze enemies.</t>
+          <t>Stevie heals from his own attacks.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Thunderstones</t>
+          <t>Human Pinball</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -3254,63 +3160,63 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink, Pocket Rocks</t>
+          <t>Repulsion Ink, Helmet</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Stevie's rocks chain lightning and burst sparks from Electric Ink walls.</t>
+          <t>Contact explosions knock nearby enemies away from Stevie.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Stevie the Unreasonable</t>
+          <t>THE STORM</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Two-part synergy</t>
+          <t>Major build</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink, Stevie Has Had Enough</t>
+          <t>Electric Ink, Frost Ink, Gravity Ink</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Stevie heals from his own attacks.</t>
+          <t>Gravity clusters, frost holds, lightning shreds the whole pack.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Human Pinball</t>
+          <t>INFERNO</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Two-part synergy</t>
+          <t>Major build</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink, Helmet</t>
+          <t>Fire Ink, Blast Ink, Repulsion Ink</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Contact explosions knock nearby enemies away from Stevie.</t>
+          <t>Burning explosions hurl ordinary monsters farther, with harder landings and a 1.6s stun; leave stronger four-second fire patches. Bosses resist launches.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>THE STORM</t>
+          <t>THE BLACK HOLE</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -3320,19 +3226,19 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink, Frost Ink, Gravity Ink</t>
+          <t>Gravity Ink, Void Ink, Closed Loop</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Gravity clusters, frost holds, lightning shreds the whole pack.</t>
+          <t>Closed loops become miniature event horizons.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>INFERNO</t>
+          <t>NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -3342,19 +3248,19 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink, Blast Ink, Repulsion Ink</t>
+          <t>Poison Ink, Vampire Ink, Gravity Ink</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Burning explosions hurl ordinary monsters farther, with harder landings and a 1.6s stun; leave stronger four-second fire patches. Bosses resist launches.</t>
+          <t>Pinned poisoned enemies continuously feed Stevie health.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>THE BLACK HOLE</t>
+          <t>TESLA CAGE</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -3364,76 +3270,10 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink, Void Ink, Closed Loop</t>
+          <t>Electric Ink, Architect, Closed Loop</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Closed loops become miniature event horizons.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="88" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>NECROTIC ENGINE</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Major build</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Poison Ink, Vampire Ink, Gravity Ink</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>Pinned poisoned enemies continuously feed Stevie health.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="88" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>ABSOLUTE ZERO</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Major build</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Frost Ink, Repulsion Ink, Double Stroke (or Triple Stroke)</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Parallel walls become freezing launch rails.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="88" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>TESLA CAGE</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Major build</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>Electric Ink, Architect, Closed Loop</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Closed intersecting geometry becomes a powered electric circuit.</t>
         </is>
@@ -4586,7 +4426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5052,7 +4892,7 @@
     <row r="14" ht="88" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Double Stroke</t>
+          <t>Doodle Stitch</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -5062,20 +4902,24 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Each stroke adds a parallel wall with 60% of the original durability.</t>
+          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Implemented replacement</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Replaces Quick Sketch. Playtest endpoint reach, the three diminishing HP additions, damaged-wall rescue and fourth-plus extensions without new HP.</t>
+        </is>
+      </c>
       <c r="G14" s="4" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr"/>
@@ -5084,34 +4928,30 @@
     <row r="15" ht="88" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Doodle Stitch</t>
+          <t>Patch Job</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
+          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Implemented replacement</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Replaces Quick Sketch. Playtest endpoint reach, the three diminishing HP additions, damaged-wall rescue and fourth-plus extensions without new HP.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr"/>
@@ -5120,30 +4960,34 @@
     <row r="16" ht="88" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Patch Job</t>
+          <t>Freehand</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
+          <t>Spend 80 real ink to charge a limited free-ink bank. Stacking increases the free bank.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Check whether the charge threshold and bank are understood; strengthen the ready-state cue before changing the economy.</t>
+        </is>
+      </c>
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
@@ -5152,7 +4996,7 @@
     <row r="17" ht="88" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Freehand</t>
+          <t>Living Fountain Pen</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -5162,24 +5006,20 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Spend 80 real ink to charge a limited free-ink bank. Stacking increases the free bank.</t>
+          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Check whether the charge threshold and bank are understood; strengthen the ready-state cue before changing the economy.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="4" t="inlineStr"/>
       <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr"/>
@@ -5188,7 +5028,7 @@
     <row r="18" ht="88" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Living Fountain Pen</t>
+          <t>Bottomless Pen</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -5198,7 +5038,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
+          <t>Per level: +40 max ink and +2 ink/s at first, with smaller regeneration bonuses on repeats.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -5220,17 +5060,17 @@
     <row r="19" ht="88" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Triple Stroke</t>
+          <t>Fortress Geometry</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Every stroke adds TWO parallel walls, each with 60% durability.</t>
+          <t>Per level: +50% closed-shape durability. Shares Closed Loop’s diminishing ink refund, completion repair and enclosed-enemy damage bonus (15% / 15% / 10% at the first utility level).</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -5252,30 +5092,34 @@
     <row r="20" ht="88" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Bottomless Pen</t>
+          <t>Bandages</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Stevie / rocks / survival</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Per level: +40 max ink and +2 ink/s at first, with smaller regeneration bonuses on repeats.</t>
+          <t>Heal 8 extra HP between waves.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Compare between-wave healing with instant healing and kill healing; consider a useful full-health benefit if it is consistently passed over.</t>
+        </is>
+      </c>
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
@@ -5284,17 +5128,17 @@
     <row r="21" ht="88" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Fortress Geometry</t>
+          <t>Helmet</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Stevie / rocks / survival</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Per level: +50% closed-shape durability. Shares Closed Loop’s diminishing ink refund, completion repair and enclosed-enemy damage bonus (15% / 15% / 10% at the first utility level).</t>
+          <t>Stevie takes 10% less contact damage.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -5316,7 +5160,7 @@
     <row r="22" ht="88" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Bandages</t>
+          <t>Pocket Rocks</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -5326,24 +5170,20 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Heal 8 extra HP between waves.</t>
+          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Compare between-wave healing with instant healing and kill healing; consider a useful full-health benefit if it is consistently passed over.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="4" t="inlineStr"/>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr"/>
@@ -5352,7 +5192,7 @@
     <row r="23" ht="88" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Helmet</t>
+          <t>Better Rocks</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -5362,7 +5202,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Stevie takes 10% less contact damage.</t>
+          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -5384,7 +5224,7 @@
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Pocket Rocks</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -5394,7 +5234,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
+          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -5416,7 +5256,7 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Better Rocks</t>
+          <t>Really Good Rocks</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -5426,7 +5266,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -5448,7 +5288,7 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -5458,7 +5298,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -5480,17 +5320,17 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Really Good Rocks</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -5512,17 +5352,17 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Stevie Has Had Enough</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -5544,7 +5384,7 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -5554,20 +5394,24 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
+        </is>
+      </c>
       <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr"/>
@@ -5576,7 +5420,7 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -5586,7 +5430,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -5608,34 +5452,30 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Ink effects</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr"/>
@@ -5644,17 +5484,17 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Ink effects</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -5676,7 +5516,7 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -5686,7 +5526,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -5708,7 +5548,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -5718,7 +5558,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5740,7 +5580,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -5750,7 +5590,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -5772,7 +5612,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -5782,7 +5622,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -5804,7 +5644,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -5814,7 +5654,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -5836,7 +5676,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -5846,20 +5686,24 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
+        </is>
+      </c>
       <c r="G38" s="4" t="inlineStr"/>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr"/>
@@ -5868,7 +5712,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -5878,7 +5722,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -5900,7 +5744,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -5910,24 +5754,20 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="4" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr"/>
@@ -5936,7 +5776,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Death Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -5946,7 +5786,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -5965,77 +5805,13 @@
       <c r="I41" s="4" t="inlineStr"/>
       <c r="J41" s="4" t="inlineStr"/>
     </row>
-    <row r="42" ht="88" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Chaos Ink</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Ink effects</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Not rated</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="4" t="inlineStr"/>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr"/>
-      <c r="J42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43" ht="88" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Death Ink</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Ink effects</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Not rated</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="4" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G43" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
+    <dataValidation sqref="G2:G41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Keep,Rework,Remove,Test first"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add timed erase trips, readable spark gaps and local firebreaks
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.22</t>
+          <t>Alpha 0.1.23</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Erase small hostile pencils/spikes, sacrificing return damage. Erasing paid electric ink between surviving wall ends discharges up to 12 + 2 × Electric Ink level damage, limited to 0.8 × removed paid ink, with a 0.8-second wall cooldown retained by fragments. Erase Chonks’s recovery support or Boingus’s fresh rebound support to stun for 1.4 seconds; each monster has a 6-second stumble cooldown.</t>
+          <t>Erase small hostile pencils/spikes, sacrificing return damage. Erasing paid electric ink between surviving wall ends discharges up to 12 + 2 × Electric Ink level damage, limited to 0.8 × removed paid ink, with a 0.8-second wall cooldown retained by fragments. Erase Chonks’s recovery support or Boingus’s fresh rebound support to stun for 1.4 seconds; each monster has a 6-second stumble cooldown. Trip Line: erase a wall within 0.45 seconds of Crash Dash or a moving Chonks reaching it to earn a safe skid and 1.4-second stumble. Bosses and airborne enemies are excluded. Firebreak: erase strips through existing Napalm/Plaguefire patches; cleared ground remains excluded from that patch’s visuals and damage, including later growth. New patches can reignite it.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Polish early paper tearing, Dash size and boss entrance celebrations
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.24</t>
+          <t>Alpha 0.1.25</t>
         </is>
       </c>
     </row>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>About 2 seconds of local active eraser rubbing tears a hole. Each wave starts with fresh paper; wear and holes reset, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
+          <t>About 1 second of local active eraser rubbing tears a hole. Each wave starts with fresh paper; wear and holes reset, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Retune paper-ball damage and improve ink regen, HUD and eraser sizing
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.27</t>
+          <t>Alpha 0.1.38</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1694,17 +1694,17 @@
     <row r="22" ht="88" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Pocket Rocks</t>
+          <t>Paper Balls</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
+          <t>Unlock paper-ball throwing. Starts near 2 damage; repeat picks and stronger builds gain less, approaching 30 base damage. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1724,14 +1724,10 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Hot Rocks, Snowball Fight, Thunderstones</t>
-        </is>
-      </c>
+          <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1741,17 +1737,17 @@
     <row r="23" ht="88" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Better Rocks</t>
+          <t>Tightly Crumpled</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1771,7 +1767,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1789,7 +1785,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1827,17 +1823,17 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Really Good Rocks</t>
+          <t>Perfect Paper Balls</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>A stronger paper-ball damage boost, with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1857,7 +1853,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
@@ -1875,12 +1871,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1900,7 +1896,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2124,7 +2120,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Rocks, INFERNO</t>
+          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2312,7 +2308,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunderstones, THE STORM, TESLA CAGE</t>
+          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -3062,7 +3058,7 @@
     <row r="21" ht="88" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Hot Rocks</t>
+          <t>Hot Paper</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -3072,12 +3068,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink, Pocket Rocks</t>
+          <t>Fire Ink, Paper Balls</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Stevie's rocks ignite enemies.</t>
+          <t>Stevie's paper balls ignite enemies.</t>
         </is>
       </c>
     </row>
@@ -3094,19 +3090,19 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink, Pocket Rocks</t>
+          <t>Frost Ink, Paper Balls</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Stevie's rocks chill and sometimes freeze enemies.</t>
+          <t>Stevie's paper balls chill and sometimes freeze enemies.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="88" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Thunderstones</t>
+          <t>Thunder Paper</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -3116,12 +3112,12 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink, Pocket Rocks</t>
+          <t>Electric Ink, Paper Balls</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Stevie's rocks chain lightning and burst sparks from Electric Ink walls.</t>
+          <t>Stevie's paper balls chain lightning and burst sparks from Electric Ink walls.</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3592,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Start throwing crumpled paper: 3 damage per rank. Higher ranks throw a little faster.</t>
+          <t>Start throwing crumpled paper: 2 damage per rank. Higher ranks throw a little faster.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -3609,12 +3605,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>3 starting paper-ball damage · 1.5s between throws</t>
+          <t>2 starting paper-ball damage · 1.5s between throws</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>9 starting paper-ball damage · 1.3s between throws</t>
+          <t>6 starting paper-ball damage · 1.3s between throws</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -4283,7 +4279,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>About 1 second of local active eraser rubbing tears a hole. Each wave starts with fresh paper; wear and holes reset, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; rocks still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
+          <t>About 1 second of local active eraser rubbing tears a hole. Each wave starts with fresh paper; wear and holes reset, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; paper balls still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -4334,7 +4330,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Unlocked through throwing upgrades, Paper Ball Practice or a Doodle Scrap discovery. Automatically targets a nearby enemy within 210 pixels before range notes. Desktop WASD steers throws while held; releasing restores auto-aim. Touch keeps auto-aim. Damage and rate grow with investment; Pocket Rocks also unlocks rock/ink synergies.</t>
+          <t>Unlocked through throwing upgrades, Paper Ball Practice or a Doodle Scrap discovery. Automatically targets a nearby enemy within 210 pixels before range notes. Desktop WASD steers throws while held; releasing restores auto-aim. Touch keeps auto-aim. Base paper-ball damage gains diminish toward 30; notebook practice adds 2 starting damage per rank, and discovery alone starts at 2. Doodle Notes add behaviors and may increase individual projectile damage. Paper Balls also unlocks paper/ink synergies.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -4597,7 +4593,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -5097,7 +5093,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -5133,7 +5129,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -5160,17 +5156,17 @@
     <row r="22" ht="88" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Pocket Rocks</t>
+          <t>Paper Balls</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Unlock rock throwing: +4 first-level damage, later gains grow to +9. Throws every 1.6s; preserves faster throws.</t>
+          <t>Unlock paper-ball throwing. Starts near 2 damage; repeat picks and stronger builds gain less, approaching 30 base damage. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -5192,17 +5188,17 @@
     <row r="23" ht="88" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Better Rocks</t>
+          <t>Tightly Crumpled</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>+6 first-level rock damage, later gains grow to +12. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -5229,7 +5225,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -5256,17 +5252,17 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Really Good Rocks</t>
+          <t>Perfect Paper Balls</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+12 first-level rock damage, later gains grow to +24. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>A stronger paper-ball damage boost, with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -5293,12 +5289,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Stevie / rocks / survival</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>+8 first-level rock damage, later gains grow to +15. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Give Black Ice skating, crowd bumps and spin-out animations
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.38</t>
+          <t>Alpha 0.1.41</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Frozen enemies are shoved harder and stay slowed.</t>
+          <t>Repelling frozen monsters sends them skating into their friends before a spin-out. Bosses resist the slide.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Turn Thermal Shock into a pressure-cooker steam reaction
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.41</t>
+          <t>Alpha 0.1.42</t>
         </is>
       </c>
     </row>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Burning frozen enemies crack for burst damage and stun.</t>
+          <t>Fire heats a frozen monster into a pressure bomb: glowing cracks, then a steam pop consumes fire and freeze, damages it and briefly staggers nearby monsters. Bosses resist staggering.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make Rail Ink radiate electric surges amplified by paper hits
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.42</t>
+          <t>Alpha 0.1.43</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Repelled enemies become charged and zap nearby targets.</t>
+          <t>Repelled monsters radiate a small electric surge. Electric paper-ball hits widen the active field and send fresh ripples; overlapping surges share a hit cooldown.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unlock circle enclosures and temporary paper-ball turrets after wave ten
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -216,8 +216,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G11" headerRowCount="1">
-  <autoFilter ref="A1:G11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G12" headerRowCount="1">
+  <autoFilter ref="A1:G12"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Perk"/>
     <tableColumn id="2" name="Current ability"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.60</t>
+          <t>Alpha 0.1.61</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" ht="88" customHeight="1">
@@ -3290,7 +3290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3342,12 +3342,12 @@
     <row r="2" ht="88" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Starter Eraser</t>
+          <t>Circle Studies</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Stevie’s free first purchase. Adds 5 percentage points to ink recovery when erasing; applies to every new run.</t>
+          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -3355,17 +3355,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>+5% erase recovery · permanent</t>
+          <t>Enclosures and paper turrets · permanent</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>+5% erase recovery · permanent</t>
+          <t>Enclosures and paper turrets · permanent</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -3377,12 +3377,12 @@
     <row r="3" ht="88" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Doodle Scraps</t>
+          <t>Starter Eraser</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Unlock mysterious paper drops in future runs, from any wave. Draw through one and choose a stacking trick for Stevie’s paper balls. Discover elemental throws, wall rides, decoys and Connect the Dots. Finds last only for that run.</t>
+          <t>Stevie’s free first purchase. Adds 5 percentage points to ink recovery when erasing; applies to every new run.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -3390,17 +3390,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Doodle Scraps can drop from wave 1</t>
+          <t>+5% erase recovery · permanent</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Doodle Scraps can drop from wave 1</t>
+          <t>+5% erase recovery · permanent</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -3412,30 +3412,30 @@
     <row r="4" ht="88" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Your Drawing Tool</t>
+          <t>Doodle Scraps</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Grow from Pencil to Mechanical Pencil (rank 3), Simple Pen (rank 6), and Scented Sharpie (rank 10). Every rank has its own artwork and adds +8 base wall HP. Pens unlock a third effect slot; Sharpies unlock a fourth.</t>
+          <t>Unlock mysterious paper drops in future runs, from any wave. Draw through one and choose a stacking trick for Stevie’s paper balls. Discover elemental throws, wall rides, decoys and Connect the Dots. Finds last only for that run.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>5, 8, 12, 16, 20, 24, 30, 36, 44, 55</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Pencil · 2 effect slots · +8 base wall HP</t>
+          <t>Doodle Scraps can drop from wave 1</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Scented Sharpie · 4 effect slots · +80 base wall HP</t>
+          <t>Doodle Scraps can drop from wave 1</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -3447,30 +3447,30 @@
     <row r="5" ht="88" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bigger Starting Tank</t>
+          <t>Your Drawing Tool</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>+20 starting/max ink per rank.</t>
+          <t>Grow from Pencil to Mechanical Pencil (rank 3), Simple Pen (rank 6), and Scented Sharpie (rank 10). Every rank has its own artwork and adds +8 base wall HP. Pens unlock a third effect slot; Sharpies unlock a fourth.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24, 40, 60</t>
+          <t>5, 8, 12, 16, 20, 24, 30, 36, 44, 55</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>+20 starting/max ink</t>
+          <t>Pencil · 2 effect slots · +8 base wall HP</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>+100 starting/max ink</t>
+          <t>Scented Sharpie · 4 effect slots · +80 base wall HP</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3482,30 +3482,30 @@
     <row r="6" ht="88" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Refill Practice</t>
+          <t>Bigger Starting Tank</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+1 starting ink regeneration per second per rank. Stacks with run upgrades.</t>
+          <t>+20 starting/max ink per rank.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24</t>
+          <t>5, 12, 24, 40, 60</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>+1 starting ink/s</t>
+          <t>+20 starting/max ink</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>+3 starting ink/s</t>
+          <t>+100 starting/max ink</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -3517,30 +3517,30 @@
     <row r="7" ht="88" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Extra Credit</t>
+          <t>Refill Practice</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Start every run with four reward choices instead of three. Boss rewards already have four.</t>
+          <t>+1 starting ink regeneration per second per rank. Stacks with run upgrades.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>5, 12, 24</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>4 reward choices from the first wave</t>
+          <t>+1 starting ink/s</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>4 reward choices from the first wave</t>
+          <t>+3 starting ink/s</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -3552,30 +3552,30 @@
     <row r="8" ht="88" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lunchbox Band-Aids</t>
+          <t>Extra Credit</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>+8 starting/max Stevie HP per rank.</t>
+          <t>Start every run with four reward choices instead of three. Boss rewards already have four.</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24, 40</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>+8 Stevie HP</t>
+          <t>4 reward choices from the first wave</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>+32 Stevie HP</t>
+          <t>4 reward choices from the first wave</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -3587,30 +3587,30 @@
     <row r="9" ht="88" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Paper Ball Practice</t>
+          <t>Lunchbox Band-Aids</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Start throwing crumpled paper: 2 damage per rank. Higher ranks throw a little faster.</t>
+          <t>+8 starting/max Stevie HP per rank.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24</t>
+          <t>5, 12, 24, 40</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2 starting paper-ball damage · 1.5s between throws</t>
+          <t>+8 Stevie HP</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>6 starting paper-ball damage · 1.3s between throws</t>
+          <t>+32 Stevie HP</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3622,30 +3622,30 @@
     <row r="10" ht="88" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lunch Money</t>
+          <t>Paper Ball Practice</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+          <t>Start throwing crumpled paper: 2 damage per rank. Higher ranks throw a little faster.</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>5, 12</t>
+          <t>5, 12, 24</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>+1 starting rerolls</t>
+          <t>2 starting paper-ball damage · 1.5s between throws</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>+2 starting rerolls</t>
+          <t>6 starting paper-ball damage · 1.3s between throws</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -3657,33 +3657,68 @@
     <row r="11" ht="88" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Lunch Money</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>5, 12</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting rerolls</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>+2 starting rerolls</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>js/notebook.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="88" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>Lucky Eraser</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>+2 starting Luck per rank, improving upgrade rarity odds.</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C12" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>5, 12, 24, 40</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>+2 starting Luck</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>+8 starting Luck</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>js/notebook.js</t>
         </is>

</xml_diff>

<commit_message>
Disable paper turrets throughout boss waves
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.61</t>
+          <t>Alpha 0.1.62</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate.</t>
+          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. Turrets are unavailable on boss waves.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">

</xml_diff>

<commit_message>
Allow new paper turrets to replace the existing cannon
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.63</t>
+          <t>Alpha 0.1.64</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. Turrets are unavailable on boss waves.</t>
+          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. A new turret replaces the old one. Turrets are unavailable on boss waves.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">

</xml_diff>

<commit_message>
Add permanent turret branches and support three active cannons
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -216,8 +216,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G12" headerRowCount="1">
-  <autoFilter ref="A1:G12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G17" headerRowCount="1">
+  <autoFilter ref="A1:G17"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Perk"/>
     <tableColumn id="2" name="Current ability"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.67</t>
+          <t>Alpha 0.1.68</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" ht="88" customHeight="1">
@@ -3290,7 +3290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. A new turret replaces the old one. Turrets are unavailable on boss waves.</t>
+          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. The turret branch improves range, duration, capacity, firing rate and build time. A new turret replaces the oldest when your capacity is full. Turrets are unavailable on boss waves.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -3377,30 +3377,30 @@
     <row r="3" ht="88" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Starter Eraser</t>
+          <t>Long Paper Barrel</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Stevie’s free first purchase. Adds 5 percentage points to ink recovery when erasing; applies to every new run.</t>
+          <t>After Circle Studies: +30 turret targeting range per rank, from 210 to 300. Doodle Note range bonuses still belong to Stevie.</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10, 20, 35</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>+5% erase recovery · permanent</t>
+          <t>240 turret range</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>+5% erase recovery · permanent</t>
+          <t>300 turret range</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -3412,30 +3412,30 @@
     <row r="4" ht="88" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Doodle Scraps</t>
+          <t>Stubborn Folds</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Unlock mysterious paper drops in future runs, from any wave. Draw through one and choose a stacking trick for Stevie’s paper balls. Discover elemental throws, wall rides, decoys and Connect the Dots. Finds last only for that run.</t>
+          <t>After Circle Studies: +3 seconds per turret per rank, from 10 to 19 seconds. Replacement always starts a fresh lifetime.</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>10, 20, 35</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Doodle Scraps can drop from wave 1</t>
+          <t>13 seconds per turret</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Doodle Scraps can drop from wave 1</t>
+          <t>19 seconds per turret</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -3447,30 +3447,30 @@
     <row r="5" ht="88" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Your Drawing Tool</t>
+          <t>Cannon Club</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Grow from Pencil to Mechanical Pencil (rank 3), Simple Pen (rank 6), and Scented Sharpie (rank 10). Every rank has its own artwork and adds +8 base wall HP. Pens unlock a third effect slot; Sharpies unlock a fourth.</t>
+          <t>After Circle Studies: +1 active turret per rank, up to three. Building beyond your limit crumbles the oldest cannon.</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>5, 8, 12, 16, 20, 24, 30, 36, 44, 55</t>
+          <t>30, 60</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Pencil · 2 effect slots · +8 base wall HP</t>
+          <t>2 active turrets</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Scented Sharpie · 4 effect slots · +80 base wall HP</t>
+          <t>3 active turrets</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3482,30 +3482,30 @@
     <row r="6" ht="88" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Bigger Starting Tank</t>
+          <t>Busy Barrels</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>+20 starting/max ink per rank.</t>
+          <t>After Long Paper Barrel: reduce turret firing interval by 0.1 seconds per rank, from 1.25 to 0.95 seconds. Doodle Note throw-speed bonuses still belong to Stevie.</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24, 40, 60</t>
+          <t>10, 20, 35</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>+20 starting/max ink</t>
+          <t>1.15 seconds between turret shots</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>+100 starting/max ink</t>
+          <t>0.95 seconds between turret shots</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -3517,30 +3517,30 @@
     <row r="7" ht="88" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Refill Practice</t>
+          <t>Quick Origami</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>+1 starting ink regeneration per second per rank. Stacks with run upgrades.</t>
+          <t>After Stubborn Folds: shorten the automatic build wait by one second per rank, from three to one. You can still confirm or cancel immediately.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24</t>
+          <t>15, 30</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>+1 starting ink/s</t>
+          <t>2 seconds to auto-build</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>+3 starting ink/s</t>
+          <t>1 second to auto-build</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -3552,12 +3552,12 @@
     <row r="8" ht="88" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Extra Credit</t>
+          <t>Starter Eraser</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Start every run with four reward choices instead of three. Boss rewards already have four.</t>
+          <t>Stevie’s free first purchase. Adds 5 percentage points to ink recovery when erasing; applies to every new run.</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -3565,17 +3565,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>4 reward choices from the first wave</t>
+          <t>+5% erase recovery · permanent</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>4 reward choices from the first wave</t>
+          <t>+5% erase recovery · permanent</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -3587,30 +3587,30 @@
     <row r="9" ht="88" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Lunchbox Band-Aids</t>
+          <t>Doodle Scraps</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>+8 starting/max Stevie HP per rank.</t>
+          <t>Unlock mysterious paper drops in future runs, from any wave. Draw through one and choose a stacking trick for Stevie’s paper balls. Discover elemental throws, wall rides, decoys and Connect the Dots. Finds last only for that run.</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24, 40</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>+8 Stevie HP</t>
+          <t>Doodle Scraps can drop from wave 1</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>+32 Stevie HP</t>
+          <t>Doodle Scraps can drop from wave 1</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -3622,30 +3622,30 @@
     <row r="10" ht="88" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Paper Ball Practice</t>
+          <t>Your Drawing Tool</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Start throwing crumpled paper: 2 damage per rank. Higher ranks throw a little faster.</t>
+          <t>Grow from Pencil to Mechanical Pencil (rank 3), Simple Pen (rank 6), and Scented Sharpie (rank 10). Every rank has its own artwork and adds +8 base wall HP. Pens unlock a third effect slot; Sharpies unlock a fourth.</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24</t>
+          <t>5, 8, 12, 16, 20, 24, 30, 36, 44, 55</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2 starting paper-ball damage · 1.5s between throws</t>
+          <t>Pencil · 2 effect slots · +8 base wall HP</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>6 starting paper-ball damage · 1.3s between throws</t>
+          <t>Scented Sharpie · 4 effect slots · +80 base wall HP</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -3657,30 +3657,30 @@
     <row r="11" ht="88" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Lunch Money</t>
+          <t>Bigger Starting Tank</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+          <t>+20 starting/max ink per rank.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>5, 12</t>
+          <t>5, 12, 24, 40, 60</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>+1 starting rerolls</t>
+          <t>+20 starting/max ink</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>+2 starting rerolls</t>
+          <t>+100 starting/max ink</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -3692,33 +3692,208 @@
     <row r="12" ht="88" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Refill Practice</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting ink regeneration per second per rank. Stacks with run upgrades.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>5, 12, 24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting ink/s</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>+3 starting ink/s</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>js/notebook.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="88" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Extra Credit</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Start every run with four reward choices instead of three. Boss rewards already have four.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>4 reward choices from the first wave</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>4 reward choices from the first wave</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>js/notebook.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="88" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Lunchbox Band-Aids</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>+8 starting/max Stevie HP per rank.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>5, 12, 24, 40</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>+8 Stevie HP</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>+32 Stevie HP</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>js/notebook.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="88" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Paper Ball Practice</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Start throwing crumpled paper: 2 damage per rank. Higher ranks throw a little faster.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>5, 12, 24</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2 starting paper-ball damage · 1.5s between throws</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>6 starting paper-ball damage · 1.3s between throws</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>js/notebook.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="88" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Lunch Money</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>5, 12</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting rerolls</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>+2 starting rerolls</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>js/notebook.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="88" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Lucky Eraser</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>+2 starting Luck per rank, improving upgrade rarity odds.</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C17" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>5, 12, 24, 40</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>+2 starting Luck</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>+8 starting Luck</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>js/notebook.js</t>
         </is>

</xml_diff>

<commit_message>
Reduce late-wave crowds and make specialist setups call reinforcements
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.69</t>
+          <t>Alpha 0.1.70</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. The turret branch improves range, duration, capacity, firing rate and build time. A new turret replaces the oldest when your capacity is full. Turrets are unavailable on boss waves.</t>
+          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. The turret branch improves range, duration, capacity, firing rate and build time. A new turret replaces the oldest when your capacity is full. Turrets work during the timed wave and disappear when its boss enters.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">

</xml_diff>

<commit_message>
Reduce Vampire healing base and per-rank sustain
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.70</t>
+          <t>Alpha 0.1.100</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -5860,7 +5860,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact and heals for 25% of damage dealt, sharing the 6 HP/s healing budget.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add permanent opening upgrade choice and gradual turret erasure
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -185,8 +185,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I41" headerRowCount="1">
-  <autoFilter ref="A1:I41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I40" headerRowCount="1">
+  <autoFilter ref="A1:I40"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -216,8 +216,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G17" headerRowCount="1">
-  <autoFilter ref="A1:G17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="NotebookPerksTable" displayName="NotebookPerksTable" ref="A1:G18" headerRowCount="1">
+  <autoFilter ref="A1:G18"/>
   <tableColumns count="7">
     <tableColumn id="1" name="Perk"/>
     <tableColumn id="2" name="Current ability"/>
@@ -257,8 +257,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J41" headerRowCount="1">
-  <autoFilter ref="A1:J41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J40" headerRowCount="1">
+  <autoFilter ref="A1:J40"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.100</t>
+          <t>Alpha 0.1.116</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" ht="88" customHeight="1">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" ht="88" customHeight="1">
@@ -746,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -929,7 +929,11 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Heavy Artillery</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1029,17 +1033,17 @@
     <row r="7" ht="88" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Fat Marker</t>
+          <t>Lucky Scribble</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>+2 line width and +15 wall HP.</t>
+          <t>+8 Luck: improves rarity odds for future upgrades and rerolls.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1062,11 +1066,7 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Heavy Artillery</t>
-        </is>
-      </c>
+      <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1076,7 +1076,7 @@
     <row r="8" ht="88" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lucky Scribble</t>
+          <t>Clean Erasing</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>+8 Luck: improves rarity odds for future upgrades and rerolls.</t>
+          <t>Recover 10 percentage points more paid ink from healthy erased walls per level, up to 60%. Damaged walls return less; free lines and copies return nothing.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Erased paid-ink recovery capped at 60%; damaged sections return less; no free/copy refunds.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1119,7 +1119,7 @@
     <row r="9" ht="88" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Clean Erasing</t>
+          <t>Recycling</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Recover 10 percentage points more paid ink from healthy erased walls per level, up to 60%. Damaged walls return less; free lines and copies return nothing.</t>
+          <t>Kills refund 5 ink, sharing an 8 ink/s refill budget.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Erased paid-ink recovery capped at 60%; damaged sections return less; no free/copy refunds.</t>
+          <t>Shared kill-ink recovery budget: 8 ink/s.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1162,17 +1162,17 @@
     <row r="10" ht="88" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Recycling</t>
+          <t>Closed Loop</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Kills refund 5 ink, sharing an 8 ink/s refill budget.</t>
+          <t>Closed shapes gain +40% durability. First loop-utility level: 15% paid ink back, repair nearby walls by 15% of missing HP, and +10% damage inside. Later levels have diminishing gains; repair is capped by ink spent.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1192,10 +1192,14 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Shared kill-ink recovery budget: 8 ink/s.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
+          <t>Shares diminishing loop utility with Fortress Geometry; refunds/repair depend on paid ink; utility overlaps do not stack.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Gravity Trap, Ring of Fire, THE BLACK HOLE, TESLA CAGE</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1205,7 +1209,7 @@
     <row r="11" ht="88" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Closed Loop</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1215,7 +1219,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Closed shapes gain +40% durability. First loop-utility level: 15% paid ink back, repair nearby walls by 15% of missing HP, and +10% damage inside. Later levels have diminishing gains; repair is capped by ink spent.</t>
+          <t>Each wall intersection adds 15% durability.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1235,12 +1239,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Shares diminishing loop utility with Fortress Geometry; refunds/repair depend on paid ink; utility overlaps do not stack.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Gravity Trap, Ring of Fire, THE BLACK HOLE, TESLA CAGE</t>
+          <t>Circuit Board, Demolition Grid, TESLA CAGE</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1252,7 +1256,7 @@
     <row r="12" ht="88" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Patchwork</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1262,7 +1266,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Each wall intersection adds 15% durability.</t>
+          <t>Drawing across an old wall repairs 18 HP.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1287,7 +1291,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Circuit Board, Demolition Grid, TESLA CAGE</t>
+          <t>Blood Patch</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1299,44 +1303,40 @@
     <row r="13" ht="88" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Patchwork</t>
+          <t>Doodle Stitch</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Drawing across an old wall repairs 18 HP.</t>
+          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Blood Patch</t>
-        </is>
-      </c>
+          <t>Endpoint snap reach 16px. New-length HP: 75%, 50%, 25%, then zero. Existing damage, oldest lifetime and summed group histories are preserved; erasing retains history.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1346,37 +1346,37 @@
     <row r="14" ht="88" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Doodle Stitch</t>
+          <t>Patch Job</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
+          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Endpoint snap reach 16px. New-length HP: 75%, 50%, 25%, then zero. Existing damage, oldest lifetime and summed group histories are preserved; erasing retains history.</t>
+          <t>Shared repair-on-kill budget: 12 wall HP/s across all walls.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1389,17 +1389,17 @@
     <row r="15" ht="88" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Patch Job</t>
+          <t>Freehand</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
+          <t>Spend 80 real ink to charge a limited free-ink bank. Stacking increases the free bank.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Shared repair-on-kill budget: 12 wall HP/s across all walls.</t>
+          <t>Charges from real paid ink, not free strokes/copies; threshold 80; initial bank 40, +20 per extra level.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -1432,7 +1432,7 @@
     <row r="16" ht="88" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Freehand</t>
+          <t>Living Fountain Pen</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Spend 80 real ink to charge a limited free-ink bank. Stacking increases the free bank.</t>
+          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Charges from real paid ink, not free strokes/copies; threshold 80; initial bank 40, +20 per extra level.</t>
+          <t>Repeat level n multiplies regeneration by 1 + 0.35 / (1 + 0.5 × (n−1)).</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1475,7 +1475,7 @@
     <row r="17" ht="88" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Living Fountain Pen</t>
+          <t>Bottomless Pen</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
+          <t>Per level: +40 max ink and +2 ink/s at first, with smaller regeneration bonuses on repeats.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Repeat level n multiplies regeneration by 1 + 0.35 / (1 + 0.5 × (n−1)).</t>
+          <t>Each level adds 40 max ink; regeneration repeats use 2 / (1 + 0.4 × (n−1)).</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1518,17 +1518,17 @@
     <row r="18" ht="88" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Bottomless Pen</t>
+          <t>Fortress Geometry</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Per level: +40 max ink and +2 ink/s at first, with smaller regeneration bonuses on repeats.</t>
+          <t>Per level: +50% closed-shape durability. Shares Closed Loop’s diminishing ink refund, completion repair and enclosed-enemy damage bonus (15% / 15% / 10% at the first utility level).</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Each level adds 40 max ink; regeneration repeats use 2 / (1 + 0.4 × (n−1)).</t>
+          <t>Shares diminishing loop utility with Closed Loop; free strokes/copies do not earn ink refunds.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -1561,17 +1561,17 @@
     <row r="19" ht="88" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Fortress Geometry</t>
+          <t>Bandages</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Per level: +50% closed-shape durability. Shares Closed Loop’s diminishing ink refund, completion repair and enclosed-enemy damage bonus (15% / 15% / 10% at the first utility level).</t>
+          <t>Heal 8 extra HP between waves.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Shares diminishing loop utility with Closed Loop; free strokes/copies do not earn ink refunds.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1604,7 +1604,7 @@
     <row r="20" ht="88" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Bandages</t>
+          <t>Helmet</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Heal 8 extra HP between waves.</t>
+          <t>Stevie takes 10% less contact damage.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1634,10 +1634,14 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>Damage reduction capped at 55%; awarded levels respect remaining cap.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Human Pinball</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1647,7 +1651,7 @@
     <row r="21" ht="88" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Helmet</t>
+          <t>Paper Balls</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1657,7 +1661,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Stevie takes 10% less contact damage.</t>
+          <t>Unlock paper-ball throwing. Starts near 2 damage; repeat picks and stronger builds gain less, approaching 30 base damage. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1677,14 +1681,10 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Damage reduction capped at 55%; awarded levels respect remaining cap.</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Human Pinball</t>
-        </is>
-      </c>
+          <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1694,7 +1694,7 @@
     <row r="22" ht="88" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Paper Balls</t>
+          <t>Tightly Crumpled</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Unlock paper-ball throwing. Starts near 2 damage; repeat picks and stronger builds gain less, approaching 30 base damage. Throws every 1.6s; preserves faster throws.</t>
+          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1737,7 +1737,7 @@
     <row r="23" ht="88" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Tightly Crumpled</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
+          <t>Shared combat-healing budget: 6 HP/s.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1780,7 +1780,7 @@
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>Perfect Paper Balls</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>A stronger paper-ball damage boost, with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s.</t>
+          <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -1823,7 +1823,7 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Perfect Paper Balls</t>
+          <t>Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>A stronger paper-ball damage boost, with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1856,7 +1856,11 @@
           <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Stevie the Unreasonable</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1866,44 +1870,40 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Stevie Has Had Enough</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Stevie / paper balls / survival</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Base damage approaches 30 with diminishing per-rank gains; Doodle Note projectile reactions retain their own damage rules.</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Stevie the Unreasonable</t>
-        </is>
-      </c>
+          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -1913,7 +1913,7 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1923,27 +1923,27 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1956,7 +1956,7 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1966,27 +1966,27 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -1999,7 +1999,7 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
+          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -2042,40 +2042,44 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Ink effects</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
+        </is>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2085,7 +2089,7 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2095,7 +2099,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2120,7 +2124,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
+          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2132,7 +2136,7 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2142,7 +2146,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2167,7 +2171,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
+          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2179,7 +2183,7 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2189,7 +2193,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2214,7 +2218,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
+          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2226,7 +2230,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2236,7 +2240,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2261,7 +2265,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
+          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2273,7 +2277,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2283,7 +2287,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2308,7 +2312,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
+          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2320,7 +2324,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2330,7 +2334,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2350,12 +2354,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
+          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2367,7 +2371,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2377,7 +2381,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2397,12 +2401,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2414,7 +2418,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2424,7 +2428,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2449,7 +2453,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
+          <t>Event Horizon, THE BLACK HOLE</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2461,7 +2465,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2471,7 +2475,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2494,11 +2498,7 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Event Horizon, THE BLACK HOLE</t>
-        </is>
-      </c>
+      <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2508,7 +2508,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Death Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2538,54 +2538,11 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
       <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>js/upgrades.js</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="88" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Death Ink</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Ink effects</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>
@@ -3046,12 +3003,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink, Fat Marker</t>
+          <t>Blast Ink, Thick Ink</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Thicker walls create larger explosions.</t>
+          <t>Thick Ink makes Blast wall explosions larger.</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3347,7 +3304,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>After defeating wave 10 Wobblechomp, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. The turret branch improves range, duration, capacity, firing rate and build time. A new turret replaces the oldest when your capacity is full. Turrets work during the timed wave and disappear when its boss enters.</t>
+          <t>After defeating the wave 10 boss, unlock 30–140px circles. Enclose enemies for 50% stronger wall contact throughout the circle, or turn an empty circle outside the fort into one paper-ball turret for 10 seconds. Turrets deal 50% more paper damage with fixed range and firing rate. Rubble Ruff can gradually erase their reinforced paper; fading turrets keep full firing power until erased. The turret branch improves range, duration, capacity, firing rate and build time. A new turret replaces the oldest when your capacity is full. Turrets work during the timed wave and disappear when its boss enters.</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -3727,12 +3684,12 @@
     <row r="13" ht="88" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Extra Credit</t>
+          <t>Head Start</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Start every run with four reward choices instead of three. Boss rewards already have four.</t>
+          <t>Choose one Common upgrade before wave 1 of every new run. Uses your normal reward-choice count and starting rerolls. Does not consume a wave reward or a reserved Legendary offer.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -3740,17 +3697,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>4 reward choices from the first wave</t>
+          <t>Choose a Common upgrade before every run</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>4 reward choices from the first wave</t>
+          <t>Choose a Common upgrade before every run</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3762,30 +3719,30 @@
     <row r="14" ht="88" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Lunchbox Band-Aids</t>
+          <t>Extra Credit</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>+8 starting/max Stevie HP per rank.</t>
+          <t>Start every run with four reward choices instead of three. Boss rewards already have four.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24, 40</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>+8 Stevie HP</t>
+          <t>4 reward choices from the first wave</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>+32 Stevie HP</t>
+          <t>4 reward choices from the first wave</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3797,30 +3754,30 @@
     <row r="15" ht="88" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Paper Ball Practice</t>
+          <t>Lunchbox Band-Aids</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Start throwing crumpled paper: 2 damage per rank. Higher ranks throw a little faster.</t>
+          <t>+8 starting/max Stevie HP per rank.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>5, 12, 24</t>
+          <t>5, 12, 24, 40</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2 starting paper-ball damage · 1.5s between throws</t>
+          <t>+8 Stevie HP</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>6 starting paper-ball damage · 1.3s between throws</t>
+          <t>+32 Stevie HP</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3832,30 +3789,30 @@
     <row r="16" ht="88" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Lunch Money</t>
+          <t>Paper Ball Practice</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+          <t>Start throwing crumpled paper: 2 damage per rank. Higher ranks throw a little faster.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>5, 12</t>
+          <t>5, 12, 24</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>+1 starting rerolls</t>
+          <t>2 starting paper-ball damage · 1.5s between throws</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>+2 starting rerolls</t>
+          <t>6 starting paper-ball damage · 1.3s between throws</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3867,33 +3824,68 @@
     <row r="17" ht="88" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Lunch Money</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting reroll per rank. Each cleared wave still supplies a free reroll.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>5, 12</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>+1 starting rerolls</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>+2 starting rerolls</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>js/notebook.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="88" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Lucky Eraser</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>+2 starting Luck per rank, improving upgrade rarity odds.</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n">
+      <c r="C18" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>5, 12, 24, 40</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>+2 starting Luck</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>+8 starting Luck</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>js/notebook.js</t>
         </is>
@@ -4632,7 +4624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4862,17 +4854,17 @@
     <row r="7" ht="88" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Fat Marker</t>
+          <t>Lucky Scribble</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>+2 line width and +15 wall HP.</t>
+          <t>+8 Luck: improves rarity odds for future upgrades and rerolls.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -4894,7 +4886,7 @@
     <row r="8" ht="88" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lucky Scribble</t>
+          <t>Clean Erasing</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -4904,20 +4896,24 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>+8 Luck: improves rarity odds for future upgrades and rerolls.</t>
+          <t>Recover 10 percentage points more paid ink from healthy erased walls per level, up to 60%. Damaged walls return less; free lines and copies return nothing.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Compare recovered ink in real mobile runs with refill upgrades; verify that recovery is visible and the cap is understood.</t>
+        </is>
+      </c>
       <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr"/>
@@ -4926,7 +4922,7 @@
     <row r="9" ht="88" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Clean Erasing</t>
+          <t>Recycling</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -4936,24 +4932,20 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Recover 10 percentage points more paid ink from healthy erased walls per level, up to 60%. Damaged walls return less; free lines and copies return nothing.</t>
+          <t>Kills refund 5 ink, sharing an 8 ink/s refill budget.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Compare recovered ink in real mobile runs with refill upgrades; verify that recovery is visible and the cap is understood.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr"/>
       <c r="I9" s="4" t="inlineStr"/>
@@ -4962,17 +4954,17 @@
     <row r="10" ht="88" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Recycling</t>
+          <t>Closed Loop</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Kills refund 5 ink, sharing an 8 ink/s refill budget.</t>
+          <t>Closed shapes gain +40% durability. First loop-utility level: 15% paid ink back, repair nearby walls by 15% of missing HP, and +10% damage inside. Later levels have diminishing gains; repair is capped by ink spent.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -4994,7 +4986,7 @@
     <row r="11" ht="88" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Closed Loop</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -5004,20 +4996,24 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Closed shapes gain +40% durability. First loop-utility level: 15% paid ink back, repair nearby walls by 15% of missing HP, and +10% damage inside. Later levels have diminishing gains; repair is capped by ink spent.</t>
+          <t>Each wall intersection adds 15% durability.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Check if intersection bonuses and Circuit Board/Demolition Grid are noticeable; consider clearer intersection markers before changing numbers.</t>
+        </is>
+      </c>
       <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr"/>
@@ -5026,7 +5022,7 @@
     <row r="12" ht="88" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Patchwork</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -5036,7 +5032,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Each wall intersection adds 15% durability.</t>
+          <t>Drawing across an old wall repairs 18 HP.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -5051,7 +5047,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Check if intersection bonuses and Circuit Board/Demolition Grid are noticeable; consider clearer intersection markers before changing numbers.</t>
+          <t>Check whether deliberately redrawing across old walls feels worth the ink; consider clearer repair feedback or a stronger skill-based repair trigger.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr"/>
@@ -5062,32 +5058,32 @@
     <row r="13" ht="88" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Patchwork</t>
+          <t>Doodle Stitch</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Drawing across an old wall repairs 18 HP.</t>
+          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Implemented replacement</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Check whether deliberately redrawing across old walls feels worth the ink; consider clearer repair feedback or a stronger skill-based repair trigger.</t>
+          <t>Replaces Quick Sketch. Playtest endpoint reach, the three diminishing HP additions, damaged-wall rescue and fourth-plus extensions without new HP.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr"/>
@@ -5098,34 +5094,30 @@
     <row r="14" ht="88" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Doodle Stitch</t>
+          <t>Patch Job</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Snap new strokes to open wall endpoints. Connectors add 75%, 50%, then 25% of normal new-length HP; later extensions add none. Pay normal ink; old damage, oldest lifetime and extension history are preserved.</t>
+          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Implemented replacement</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Monitor</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Replaces Quick Sketch. Playtest endpoint reach, the three diminishing HP additions, damaged-wall rescue and fourth-plus extensions without new HP.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="4" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr"/>
@@ -5134,30 +5126,34 @@
     <row r="15" ht="88" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Patch Job</t>
+          <t>Freehand</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
+          <t>Spend 80 real ink to charge a limited free-ink bank. Stacking increases the free bank.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Check whether the charge threshold and bank are understood; strengthen the ready-state cue before changing the economy.</t>
+        </is>
+      </c>
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr"/>
@@ -5166,7 +5162,7 @@
     <row r="16" ht="88" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Freehand</t>
+          <t>Living Fountain Pen</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -5176,24 +5172,20 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Spend 80 real ink to charge a limited free-ink bank. Stacking increases the free bank.</t>
+          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Check whether the charge threshold and bank are understood; strengthen the ready-state cue before changing the economy.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr"/>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr"/>
@@ -5202,7 +5194,7 @@
     <row r="17" ht="88" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Living Fountain Pen</t>
+          <t>Bottomless Pen</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -5212,7 +5204,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
+          <t>Per level: +40 max ink and +2 ink/s at first, with smaller regeneration bonuses on repeats.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -5234,17 +5226,17 @@
     <row r="18" ht="88" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Bottomless Pen</t>
+          <t>Fortress Geometry</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Per level: +40 max ink and +2 ink/s at first, with smaller regeneration bonuses on repeats.</t>
+          <t>Per level: +50% closed-shape durability. Shares Closed Loop’s diminishing ink refund, completion repair and enclosed-enemy damage bonus (15% / 15% / 10% at the first utility level).</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -5266,30 +5258,34 @@
     <row r="19" ht="88" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Fortress Geometry</t>
+          <t>Bandages</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Per level: +50% closed-shape durability. Shares Closed Loop’s diminishing ink refund, completion repair and enclosed-enemy damage bonus (15% / 15% / 10% at the first utility level).</t>
+          <t>Heal 8 extra HP between waves.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Compare between-wave healing with instant healing and kill healing; consider a useful full-health benefit if it is consistently passed over.</t>
+        </is>
+      </c>
       <c r="G19" s="4" t="inlineStr"/>
       <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr"/>
@@ -5298,7 +5294,7 @@
     <row r="20" ht="88" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Bandages</t>
+          <t>Helmet</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -5308,24 +5304,20 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Heal 8 extra HP between waves.</t>
+          <t>Stevie takes 10% less contact damage.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Compare between-wave healing with instant healing and kill healing; consider a useful full-health benefit if it is consistently passed over.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
@@ -5334,7 +5326,7 @@
     <row r="21" ht="88" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Helmet</t>
+          <t>Paper Balls</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -5344,7 +5336,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Stevie takes 10% less contact damage.</t>
+          <t>Unlock paper-ball throwing. Starts near 2 damage; repeat picks and stronger builds gain less, approaching 30 base damage. Throws every 1.6s; preserves faster throws.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -5366,7 +5358,7 @@
     <row r="22" ht="88" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Paper Balls</t>
+          <t>Tightly Crumpled</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -5376,7 +5368,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Unlock paper-ball throwing. Starts near 2 damage; repeat picks and stronger builds gain less, approaching 30 base damage. Throws every 1.6s; preserves faster throws.</t>
+          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.65s.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -5398,7 +5390,7 @@
     <row r="23" ht="88" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Tightly Crumpled</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -5408,7 +5400,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.65s.</t>
+          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -5430,7 +5422,7 @@
     <row r="24" ht="88" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>Perfect Paper Balls</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -5440,7 +5432,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>A stronger paper-ball damage boost, with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.55s.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -5462,7 +5454,7 @@
     <row r="25" ht="88" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Perfect Paper Balls</t>
+          <t>Stevie Has Had Enough</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -5472,7 +5464,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>A stronger paper-ball damage boost, with diminishing gains toward 30 base damage. Each level shortens throws by 0.08s, down to 0.55s.</t>
+          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.14s, down to 0.45s.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -5494,17 +5486,17 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Stevie Has Had Enough</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Stevie / paper balls / survival</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Improve paper-ball damage with diminishing gains toward 30 base damage. Each level shortens throws by 0.14s, down to 0.45s.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -5526,7 +5518,7 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -5536,7 +5528,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -5558,7 +5550,7 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -5568,20 +5560,24 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
+        </is>
+      </c>
       <c r="G28" s="4" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr"/>
@@ -5590,7 +5586,7 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -5600,24 +5596,20 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr"/>
@@ -5626,17 +5618,17 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Ink effects</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -5658,7 +5650,7 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -5668,7 +5660,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -5690,7 +5682,7 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -5700,7 +5692,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -5722,7 +5714,7 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -5732,7 +5724,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -5754,7 +5746,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -5764,7 +5756,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5786,7 +5778,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -5796,7 +5788,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -5818,7 +5810,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -5828,7 +5820,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -5850,7 +5842,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -5860,20 +5852,24 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
+        </is>
+      </c>
       <c r="G37" s="4" t="inlineStr"/>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr"/>
@@ -5882,7 +5878,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -5892,24 +5888,20 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="4" t="inlineStr"/>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr"/>
@@ -5918,7 +5910,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -5928,7 +5920,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -5950,7 +5942,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Death Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -5960,7 +5952,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -5979,45 +5971,13 @@
       <c r="I40" s="4" t="inlineStr"/>
       <c r="J40" s="4" t="inlineStr"/>
     </row>
-    <row r="41" ht="88" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Death Ink</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Ink effects</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Not rated</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="4" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr"/>
-      <c r="J41" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
+    <dataValidation sqref="G2:G40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Keep,Rework,Remove,Test first"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add four drawing utilities with custom art and notebook wave clears
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -185,8 +185,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I40" headerRowCount="1">
-  <autoFilter ref="A1:I40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I44" headerRowCount="1">
+  <autoFilter ref="A1:I44"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -257,8 +257,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J40" headerRowCount="1">
-  <autoFilter ref="A1:J40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J44" headerRowCount="1">
+  <autoFilter ref="A1:J44"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.116</t>
+          <t>Alpha 0.1.117</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" ht="88" customHeight="1">
@@ -746,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1870,22 +1870,22 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Margin of Error</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>Erase an end of a paid, open 55–260px wall to hinge it at the other end. The next ordinary monster swings it through a safe arc, sweeping enemies away from Stevie. One hinge per wall; up to four ready gates. No ink refund for converted walls.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -1913,37 +1913,37 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Stevie's Terrible Idea</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Finish a paid, open 55–260px stroke, hold its tip still for 1 second, then release. Spend 12 extra ink to crumple it into a rolling boulder carrying your ink effects. Rolls along the stroke direction, then unfolds at half its remaining HP if room permits. 8-second cooldown; no ink refunds or repeat crumpling. Bosses resist the roll.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>legendary</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1956,22 +1956,22 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Spitball Express</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Requires permanent paper balls and Circle Studies. Allows at least two active turrets. Draw a paid line from one turret to another: the first sends its shots along it, charging them for 75% extra damage before the far turret fires. Break the line or lose either turret and the delivery stops. Draw direction sets the route.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -1999,22 +1999,22 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Red Pen Corrections</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>A red correction mark appears over an ordinary monster. Rub the mark to recruit it for 8 seconds: it throws paper balls at enemies, then runs away. One friend at a time; a new mark becomes available after 12 seconds. Bosses and specialist monsters cannot be recruited.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>legendary</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -2042,44 +2042,40 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
-        </is>
-      </c>
+          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2089,17 +2085,17 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2119,14 +2115,10 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
-        </is>
-      </c>
+          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2136,44 +2128,40 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
-        </is>
-      </c>
+          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2183,44 +2171,40 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
-        </is>
-      </c>
+          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2230,7 +2214,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2240,7 +2224,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2265,7 +2249,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
+          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2277,7 +2261,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2287,7 +2271,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2312,7 +2296,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
+          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2324,7 +2308,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2334,7 +2318,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2354,12 +2338,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2371,7 +2355,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2381,7 +2365,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2406,7 +2390,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
+          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2418,7 +2402,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2428,7 +2412,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2453,7 +2437,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Event Horizon, THE BLACK HOLE</t>
+          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2465,7 +2449,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2475,7 +2459,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2498,7 +2482,11 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
+        </is>
+      </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2508,41 +2496,225 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>Vampire Ink</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="88" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Gravity Ink</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="88" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Void Ink</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Event Horizon, THE BLACK HOLE</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="88" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Chaos Ink</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="88" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
           <t>Death Ink</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Ink effects</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>
@@ -4624,7 +4796,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5486,17 +5658,17 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Margin of Error</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>Erase an end of a paid, open 55–260px wall to hinge it at the other end. The next ordinary monster swings it through a safe arc, sweeping enemies away from Stevie. One hinge per wall; up to four ready gates. No ink refund for converted walls.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -5518,17 +5690,17 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Stevie's Terrible Idea</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Finish a paid, open 55–260px stroke, hold its tip still for 1 second, then release. Spend 12 extra ink to crumple it into a rolling boulder carrying your ink effects. Rolls along the stroke direction, then unfolds at half its remaining HP if room permits. 8-second cooldown; no ink refunds or repeat crumpling. Bosses resist the roll.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -5550,34 +5722,30 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Spitball Express</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Requires permanent paper balls and Circle Studies. Allows at least two active turrets. Draw a paid line from one turret to another: the first sends its shots along it, charging them for 75% extra damage before the far turret fires. Break the line or lose either turret and the delivery stops. Draw direction sets the route.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="4" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr"/>
@@ -5586,17 +5754,17 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Red Pen Corrections</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>A red correction mark appears over an ordinary monster. Rub the mark to recruit it for 8 seconds: it throws paper balls at enemies, then runs away. One friend at a time; a new mark becomes available after 12 seconds. Bosses and specialist monsters cannot be recruited.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -5618,17 +5786,17 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -5650,17 +5818,17 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -5682,30 +5850,34 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
+        </is>
+      </c>
       <c r="G32" s="4" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr"/>
@@ -5714,17 +5886,17 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -5746,7 +5918,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -5756,7 +5928,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5778,7 +5950,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -5788,7 +5960,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -5810,7 +5982,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -5820,7 +5992,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -5842,7 +6014,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -5852,24 +6024,20 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="4" t="inlineStr"/>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr"/>
@@ -5878,7 +6046,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -5888,7 +6056,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -5910,7 +6078,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -5920,7 +6088,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -5942,7 +6110,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Death Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -5952,7 +6120,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -5971,13 +6139,145 @@
       <c r="I40" s="4" t="inlineStr"/>
       <c r="J40" s="4" t="inlineStr"/>
     </row>
+    <row r="41" ht="88" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Gravity Ink</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Hypothesis</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42" ht="88" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Void Ink</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Not rated</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="88" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Chaos Ink</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Not rated</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="88" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Death Ink</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Not rated</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
+    <dataValidation sqref="G2:G44" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Keep,Rework,Remove,Test first"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add animated Under the Desk summon and complete combined utility update
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -185,8 +185,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I44" headerRowCount="1">
-  <autoFilter ref="A1:I44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I45" headerRowCount="1">
+  <autoFilter ref="A1:I45"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -257,8 +257,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J44" headerRowCount="1">
-  <autoFilter ref="A1:J44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J45" headerRowCount="1">
+  <autoFilter ref="A1:J45"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.117</t>
+          <t>Alpha 0.1.118</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" ht="88" customHeight="1">
@@ -746,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2042,22 +2042,22 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Under the Desk</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>Draw a paid closed shape 64–160px across, safely away from Stevie. Erase two diagonal strokes to make an X inside it. Spend 35 extra ink: a creature punches through the school desk and grabs up to three ordinary monsters within about 100px. Lasts 12 seconds; 24-second cooldown. Bosses, shielded monsters and passengers resist swallowing. The cracked wooden scar stays for the chapter. A box avoids the Circle Studies turret offer.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>legendary</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2072,7 +2072,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -2085,7 +2085,7 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2095,27 +2095,27 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -2128,7 +2128,7 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -2138,27 +2138,27 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>One-time: +1 unlock</t>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock</t>
+          <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
+          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
+          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -2214,44 +2214,40 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
-        </is>
-      </c>
+          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2261,7 +2257,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -2271,7 +2267,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2296,7 +2292,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
+          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2308,7 +2304,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2318,7 +2314,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2343,7 +2339,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
+          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2355,7 +2351,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2365,7 +2361,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2390,7 +2386,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
+          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2402,7 +2398,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2412,7 +2408,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2437,7 +2433,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
+          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2449,7 +2445,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2459,7 +2455,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2484,7 +2480,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
+          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2496,7 +2492,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2506,7 +2502,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2526,12 +2522,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2543,7 +2539,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2553,7 +2549,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2573,12 +2569,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
+          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
+          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2590,7 +2586,7 @@
     <row r="42" ht="88" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2600,7 +2596,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2625,7 +2621,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Event Horizon, THE BLACK HOLE</t>
+          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2637,7 +2633,7 @@
     <row r="43" ht="88" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2647,7 +2643,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2670,7 +2666,11 @@
           <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Event Horizon, THE BLACK HOLE</t>
+        </is>
+      </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2680,7 +2680,7 @@
     <row r="44" ht="88" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Death Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2690,7 +2690,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2710,11 +2710,54 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
       <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="88" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Death Ink</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>
@@ -4796,7 +4839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5786,17 +5829,17 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Under the Desk</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>Draw a paid closed shape 64–160px across, safely away from Stevie. Erase two diagonal strokes to make an X inside it. Spend 35 extra ink: a creature punches through the school desk and grabs up to three ordinary monsters within about 100px. Lasts 12 seconds; 24-second cooldown. Bosses, shielded monsters and passengers resist swallowing. The cracked wooden scar stays for the chapter. A box avoids the Circle Studies turret offer.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -5818,7 +5861,7 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -5828,7 +5871,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -5850,7 +5893,7 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -5860,24 +5903,20 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="4" t="inlineStr"/>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr"/>
@@ -5886,7 +5925,7 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -5896,20 +5935,24 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
+        </is>
+      </c>
       <c r="G33" s="4" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr"/>
@@ -5918,17 +5961,17 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5950,7 +5993,7 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -5960,7 +6003,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -5982,7 +6025,7 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -5992,7 +6035,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -6014,7 +6057,7 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -6024,7 +6067,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -6046,7 +6089,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -6056,7 +6099,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -6078,7 +6121,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -6088,7 +6131,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -6110,7 +6153,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -6120,7 +6163,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Destroyed walls explode and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -6142,7 +6185,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -6152,24 +6195,20 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr"/>
@@ -6178,7 +6217,7 @@
     <row r="42" ht="88" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -6188,20 +6227,24 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
+        </is>
+      </c>
       <c r="G42" s="4" t="inlineStr"/>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr"/>
@@ -6210,7 +6253,7 @@
     <row r="43" ht="88" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Void Ink</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -6220,7 +6263,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -6242,7 +6285,7 @@
     <row r="44" ht="88" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Death Ink</t>
+          <t>Chaos Ink</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -6252,7 +6295,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -6271,13 +6314,45 @@
       <c r="I44" s="4" t="inlineStr"/>
       <c r="J44" s="4" t="inlineStr"/>
     </row>
+    <row r="45" ht="88" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Death Ink</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Not rated</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G44" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
+    <dataValidation sqref="G2:G45" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Keep,Rework,Remove,Test first"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix mobile timer and direction choices; strengthen Repulsion ranks
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.118</t>
+          <t>Alpha 0.1.119</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them. Each rank pushes 10px farther.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them. Each rank pushes 10px farther.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Require half-second arming and minimum wall length for Blast
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.119</t>
+          <t>Alpha 0.1.121</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Walls at least 50px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -6163,7 +6163,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Destroyed walls explode and damage nearby enemies.</t>
+          <t>Walls at least 50px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add numbered-dot prototype and small one-time utility toys
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -185,8 +185,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I45" headerRowCount="1">
-  <autoFilter ref="A1:I45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RunUpgradesTable" displayName="RunUpgradesTable" ref="A1:I48" headerRowCount="1">
+  <autoFilter ref="A1:I48"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -257,8 +257,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J45" headerRowCount="1">
-  <autoFilter ref="A1:J45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="RetuningReviewTable" displayName="RetuningReviewTable" ref="A1:J48" headerRowCount="1">
+  <autoFilter ref="A1:J48"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Upgrade"/>
     <tableColumn id="2" name="Category"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.125</t>
+          <t>Alpha 0.1.126</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" ht="88" customHeight="1">
@@ -746,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1870,7 +1870,7 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Margin of Error</t>
+          <t>Eraser Crumbs</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Erase an end of a paid, open 55–260px wall to hinge it at the other end. The next ordinary monster swings it through a safe arc, sweeping enemies away from Stevie. One hinge per wall; up to four ready gates. No ink refund for converted walls.</t>
+          <t>Erasing 6 ink worth of your own paid walls leaves pink rubber crumbs. An ordinary monster stops to chew for 0.9 seconds. Up to three piles, lasting 8 seconds; each monster needs 5 seconds between snacks. Free walls and enemy erasing leave no crumbs.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>common</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1913,22 +1913,22 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Stevie's Terrible Idea</t>
+          <t>Please Form a Line</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Finish a paid, open 55–260px stroke, hold its tip still for 1 second, then release. Spend 12 extra ink to crumple it into a rolling boulder carrying your ink effects. Rolls along the stroke direction, then unfolds at half its remaining HP if room permits. 8-second cooldown; no ink refunds or repeat crumpling. Bosses resist the roll.</t>
+          <t>When three ordinary monsters crowd the same wall, a ONE AT A TIME sign makes two wait for 1.25 seconds while the front monster keeps chewing. Each wall has a 7-second cooldown. Bosses and specialist monsters ignore the sign.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>legendary</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1956,22 +1956,22 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Spitball Express</t>
+          <t>Connect the Dots</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Stevie / paper balls / survival</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Requires permanent paper balls and Circle Studies. Allows at least two active turrets. Draw a paid line from one turret to another: the first sends its shots along it, charging them for 75% extra damage before the far turret fires. Break the line or lose either turret and the delivery stops. Draw direction sets the route.</t>
+          <t>PROTOTYPE: defeated non-boss monsters have a 10% chance to drop numbered dots: 1, 2, 3 and onward, with no cap or expiry, even across waves. Start at 1, trace at least three numbers in order, then return to 1 in one stroke. Tracing is free. Closing clears the entire batch, including unused dots; the next drop is 1. No combat reward yet. The page shows drops and your biggest loop.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1999,22 +1999,22 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Red Pen Corrections</t>
+          <t>Margin of Error</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Stevie / paper balls / survival</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>A red correction mark appears over an ordinary monster. Rub the mark to recruit it for 8 seconds: it throws paper balls at enemies, then runs away. One friend at a time; a new mark becomes available after 12 seconds. Bosses and specialist monsters cannot be recruited.</t>
+          <t>Erase an end of a paid, open 55–260px wall to hinge it at the other end. The next ordinary monster swings it through a safe arc, sweeping enemies away from Stevie. One hinge per wall; up to four ready gates. No ink refund for converted walls.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>legendary</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2042,17 +2042,17 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Under the Desk</t>
+          <t>Stevie's Terrible Idea</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Draw a paid closed shape 64–160px across, safely away from Stevie. Erase two diagonal strokes to make an X inside it. Spend 35 extra ink: a creature punches through the school desk and grabs up to three ordinary monsters within about 100px. Lasts 12 seconds; 24-second cooldown. Bosses, shielded monsters and passengers resist swallowing. The cracked wooden scar stays for the chapter. A box avoids the Circle Studies turret offer.</t>
+          <t>Finish a paid, open 55–260px stroke, hold its tip still for 1 second, then release. Spend 12 extra ink to crumple it into a rolling boulder carrying your ink effects. Rolls along the stroke direction, then unfolds at half its remaining HP if room permits. 8-second cooldown; no ink refunds or repeat crumpling. Bosses resist the roll.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2085,22 +2085,22 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Spitball Express</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>Requires permanent paper balls and Circle Studies. Allows at least two active turrets. Draw a paid line from one turret to another: the first sends its shots along it, charging them for 75% extra damage before the far turret fires. Break the line or lose either turret and the delivery stops. Draw direction sets the route.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2115,7 +2115,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -2128,37 +2128,37 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Red Pen Corrections</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>A red correction mark appears over an ordinary monster. Rub the mark to recruit it for 8 seconds: it throws paper balls at enemies, then runs away. One friend at a time; a new mark becomes available after 12 seconds. Bosses and specialist monsters cannot be recruited.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>legendary</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -2171,22 +2171,22 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Under the Desk</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Draw a paid closed shape 64–160px across, safely away from Stevie. Erase two diagonal strokes to make an X inside it. Spend 35 extra ink: a creature punches through the school desk and grabs up to three ordinary monsters within about 100px. Lasts 12 seconds; 24-second cooldown. Bosses, shielded monsters and passengers resist swallowing. The cracked wooden scar stays for the chapter. A box avoids the Circle Studies turret offer.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare</t>
+          <t>legendary</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -2214,7 +2214,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
+          <t>One-time unlock; ordinary rewards only, no extra Legendary chances.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -2257,17 +2257,17 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2287,14 +2287,10 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
-        </is>
-      </c>
+          <t>Stored rerolls capped at 5; awarded levels respect remaining cap.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2304,44 +2300,40 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
-        </is>
-      </c>
+          <t>One-time unlock; unowned card weights multiplied by 1.8.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
       <c r="I36" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2351,44 +2343,40 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Common / Uncommon / Rare / Legendary</t>
+          <t>Common / Uncommon / Rare</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+          <t>One-time: +1 unlock</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Repeatable; caps/diminishing returns may apply</t>
+          <t>One-time unlock</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
-        </is>
-      </c>
+          <t>One-time unlock; disabled if a fourth reward choice already exists.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
       <c r="I37" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2398,7 +2386,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2408,7 +2396,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them. Each rank pushes 10px farther.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2433,7 +2421,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
+          <t>Plaguefire, Thermal Shock, Napalm Scribbles, Ring of Fire, Hot Paper, INFERNO</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2445,7 +2433,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2455,7 +2443,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2480,7 +2468,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
+          <t>Cryoshock, Black Ice, Thermal Shock, Venom Ice, Snowball Fight, THE STORM</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2492,7 +2480,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2502,7 +2490,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Walls at least 50px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2527,7 +2515,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
+          <t>Plaguefire, Leech Ink, Venom Ice, Needlepoint, NECROTIC ENGINE</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2539,7 +2527,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2549,7 +2537,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them. Each rank pushes 10px farther.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2569,12 +2557,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+          <t>See effect description and game code for per-level combat tuning.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+          <t>Black Ice, Cannon Ink, Rail Ink, Human Pinball, INFERNO</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2586,7 +2574,7 @@
     <row r="42" ht="88" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -2596,7 +2584,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2621,7 +2609,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
+          <t>Cryoshock, Tesla Well, Rail Ink, Circuit Board, Thunder Paper, THE STORM, TESLA CAGE</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2633,7 +2621,7 @@
     <row r="43" ht="88" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -2643,7 +2631,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Walls at least 50px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2668,7 +2656,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Event Horizon, THE BLACK HOLE</t>
+          <t>Singularity Ink, Cannon Ink, Napalm Scribbles, Demolition Grid, Heavy Artillery, INFERNO</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2680,7 +2668,7 @@
     <row r="44" ht="88" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2690,7 +2678,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2710,10 +2698,14 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>See effect description and game code for per-level combat tuning.</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr"/>
+          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Leech Ink, Blood Patch, Stevie the Unreasonable, NECROTIC ENGINE</t>
+        </is>
+      </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
@@ -2723,41 +2715,178 @@
     <row r="45" ht="88" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>Gravity Ink</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Singularity Ink, Tesla Well, Event Horizon, Gravity Trap, THE STORM, THE BLACK HOLE, NECROTIC ENGINE</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="88" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Void Ink</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Event Horizon, THE BLACK HOLE</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="88" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Chaos Ink</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Common / Uncommon / Rare / Legendary</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Repeatable; caps/diminishing returns may apply</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>See effect description and game code for per-level combat tuning.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>js/upgrades.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="88" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
           <t>Death Ink</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Ink effects</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Common / Uncommon / Rare / Legendary</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Common +1 / Uncommon +2 / Rare +3 / Legendary +4</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Repeatable; caps/diminishing returns may apply</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Uses an effect slot even though its per-level gain changes base wall DPS.</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr"/>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>js/upgrades.js</t>
         </is>
@@ -4839,7 +4968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5701,7 +5830,7 @@
     <row r="26" ht="88" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Margin of Error</t>
+          <t>Eraser Crumbs</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -5711,7 +5840,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Erase an end of a paid, open 55–260px wall to hinge it at the other end. The next ordinary monster swings it through a safe arc, sweeping enemies away from Stevie. One hinge per wall; up to four ready gates. No ink refund for converted walls.</t>
+          <t>Erasing 6 ink worth of your own paid walls leaves pink rubber crumbs. An ordinary monster stops to chew for 0.9 seconds. Up to three piles, lasting 8 seconds; each monster needs 5 seconds between snacks. Free walls and enemy erasing leave no crumbs.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -5733,17 +5862,17 @@
     <row r="27" ht="88" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Stevie's Terrible Idea</t>
+          <t>Please Form a Line</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Drawing / ink economy</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Finish a paid, open 55–260px stroke, hold its tip still for 1 second, then release. Spend 12 extra ink to crumple it into a rolling boulder carrying your ink effects. Rolls along the stroke direction, then unfolds at half its remaining HP if room permits. 8-second cooldown; no ink refunds or repeat crumpling. Bosses resist the roll.</t>
+          <t>When three ordinary monsters crowd the same wall, a ONE AT A TIME sign makes two wait for 1.25 seconds while the front monster keeps chewing. Each wall has a 7-second cooldown. Bosses and specialist monsters ignore the sign.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -5765,17 +5894,17 @@
     <row r="28" ht="88" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Spitball Express</t>
+          <t>Connect the Dots</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Stevie / paper balls / survival</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Requires permanent paper balls and Circle Studies. Allows at least two active turrets. Draw a paid line from one turret to another: the first sends its shots along it, charging them for 75% extra damage before the far turret fires. Break the line or lose either turret and the delivery stops. Draw direction sets the route.</t>
+          <t>PROTOTYPE: defeated non-boss monsters have a 10% chance to drop numbered dots: 1, 2, 3 and onward, with no cap or expiry, even across waves. Start at 1, trace at least three numbers in order, then return to 1 in one stroke. Tracing is free. Closing clears the entire batch, including unused dots; the next drop is 1. No combat reward yet. The page shows drops and your biggest loop.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -5797,17 +5926,17 @@
     <row r="29" ht="88" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Red Pen Corrections</t>
+          <t>Margin of Error</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Stevie / paper balls / survival</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>A red correction mark appears over an ordinary monster. Rub the mark to recruit it for 8 seconds: it throws paper balls at enemies, then runs away. One friend at a time; a new mark becomes available after 12 seconds. Bosses and specialist monsters cannot be recruited.</t>
+          <t>Erase an end of a paid, open 55–260px wall to hinge it at the other end. The next ordinary monster swings it through a safe arc, sweeping enemies away from Stevie. One hinge per wall; up to four ready gates. No ink refund for converted walls.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -5829,17 +5958,17 @@
     <row r="30" ht="88" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Under the Desk</t>
+          <t>Stevie's Terrible Idea</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Walls / shapes</t>
+          <t>Drawing / ink economy</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Draw a paid closed shape 64–160px across, safely away from Stevie. Erase two diagonal strokes to make an X inside it. Spend 35 extra ink: a creature punches through the school desk and grabs up to three ordinary monsters within about 100px. Lasts 12 seconds; 24-second cooldown. Bosses, shielded monsters and passengers resist swallowing. The cracked wooden scar stays for the chapter. A box avoids the Circle Studies turret offer.</t>
+          <t>Finish a paid, open 55–260px stroke, hold its tip still for 1 second, then release. Spend 12 extra ink to crumple it into a rolling boulder carrying your ink effects. Rolls along the stroke direction, then unfolds at half its remaining HP if room permits. 8-second cooldown; no ink refunds or repeat crumpling. Bosses resist the roll.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -5861,17 +5990,17 @@
     <row r="31" ht="88" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Loaded Deck</t>
+          <t>Spitball Express</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Future normal rewards cannot roll below Uncommon.</t>
+          <t>Requires permanent paper balls and Circle Studies. Allows at least two active turrets. Draw a paid line from one turret to another: the first sends its shots along it, charging them for 75% extra damage before the far turret fires. Break the line or lose either turret and the delivery stops. Draw direction sets the route.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -5893,17 +6022,17 @@
     <row r="32" ht="88" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Reroll Coupon</t>
+          <t>Red Pen Corrections</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Stevie / paper balls / survival</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>+2 rerolls immediately.</t>
+          <t>A red correction mark appears over an ordinary monster. Rub the mark to recruit it for 8 seconds: it throws paper balls at enemies, then runs away. One friend at a time; a new mark becomes available after 12 seconds. Bosses and specialist monsters cannot be recruited.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -5925,34 +6054,30 @@
     <row r="33" ht="88" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Collector</t>
+          <t>Under the Desk</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Rewards / recovery</t>
+          <t>Walls / shapes</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Slightly favors upgrades you have not taken yet.</t>
+          <t>Draw a paid closed shape 64–160px across, safely away from Stevie. Erase two diagonal strokes to make an X inside it. Spend 35 extra ink: a creature punches through the school desk and grabs up to three ordinary monsters within about 100px. Lasts 12 seconds; 24-second cooldown. Bosses, shielded monsters and passengers resist swallowing. The cracked wooden scar stays for the chapter. A box avoids the Circle Studies turret offer.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="4" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr"/>
@@ -5961,7 +6086,7 @@
     <row r="34" ht="88" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Greedy Goblin</t>
+          <t>Loaded Deck</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -5971,7 +6096,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Normal rewards show a fourth choice.</t>
+          <t>Future normal rewards cannot roll below Uncommon.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5993,17 +6118,17 @@
     <row r="35" ht="88" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Fire Ink</t>
+          <t>Reroll Coupon</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Wall contact ignites enemies for damage over time.</t>
+          <t>+2 rerolls immediately.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -6025,30 +6150,34 @@
     <row r="36" ht="88" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Frost Ink</t>
+          <t>Collector</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
+          <t>Slightly favors upgrades you have not taken yet.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Check whether 1.8× weighting toward unowned cards helps or disrupts a focused build; consider a more visible reward-selection benefit.</t>
+        </is>
+      </c>
       <c r="G36" s="4" t="inlineStr"/>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr"/>
@@ -6057,17 +6186,17 @@
     <row r="37" ht="88" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Poison Ink</t>
+          <t>Greedy Goblin</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Ink effects</t>
+          <t>Rewards / recovery</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Enemies build stacking poison while touching walls.</t>
+          <t>Normal rewards show a fourth choice.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -6089,7 +6218,7 @@
     <row r="38" ht="88" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Repulsion Ink</t>
+          <t>Fire Ink</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -6099,7 +6228,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them. Each rank pushes 10px farther.</t>
+          <t>Wall contact ignites enemies for damage over time.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -6121,7 +6250,7 @@
     <row r="39" ht="88" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Electric Ink</t>
+          <t>Frost Ink</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -6131,7 +6260,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
+          <t>Slows on contact from level one. Sustained contact builds a guaranteed freeze; bosses freeze for half as long.</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -6153,7 +6282,7 @@
     <row r="40" ht="88" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Blast Ink</t>
+          <t>Poison Ink</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -6163,7 +6292,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Walls at least 50px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
+          <t>Enemies build stacking poison while touching walls.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -6185,7 +6314,7 @@
     <row r="41" ht="88" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Vampire Ink</t>
+          <t>Repulsion Ink</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -6195,7 +6324,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Timed contact pulses deal impact damage, shove enemies safely away from Stevie and briefly stagger them. Each rank pushes 10px farther.</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -6217,7 +6346,7 @@
     <row r="42" ht="88" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Gravity Ink</t>
+          <t>Electric Ink</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -6227,24 +6356,20 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
+          <t>Wall contact sparks a fading chain with brief shock. Shared recovery prevents overlapping zaps; every three levels add a jump, with capped reach and targets.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Hypothesis</t>
+          <t>Not rated</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
-        </is>
-      </c>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="4" t="inlineStr"/>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr"/>
@@ -6253,7 +6378,7 @@
     <row r="43" ht="88" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Void Ink</t>
+          <t>Blast Ink</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -6263,7 +6388,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+          <t>Walls at least 50px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -6285,7 +6410,7 @@
     <row r="44" ht="88" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Chaos Ink</t>
+          <t>Vampire Ink</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -6295,7 +6420,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -6317,7 +6442,7 @@
     <row r="45" ht="88" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Death Ink</t>
+          <t>Gravity Ink</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -6327,32 +6452,132 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+          <t>Tugs nearby enemies toward wall segments without slowing movement or wall bites. Tight reach; King Doodle resists the pull, but his returnable shots bend slightly toward nearby walls.</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Not rated</t>
+          <t>Hypothesis</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Unrated</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr"/>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Measure whether enemies are held on dangerous wall segments; check readability and synergy payoff before buffing reach.</t>
+        </is>
+      </c>
       <c r="G45" s="4" t="inlineStr"/>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr"/>
       <c r="J45" s="4" t="inlineStr"/>
     </row>
+    <row r="46" ht="88" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Void Ink</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Deals steady Void damage on contact and executes weakened ordinary enemies; bosses cannot be executed.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Not rated</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr"/>
+      <c r="J46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47" ht="88" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Chaos Ink</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Sustained contact guarantees timed random ink rolls. Every roll has a working effect and extra impact damage.</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Not rated</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48" ht="88" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Death Ink</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Ink effects</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Per level: +5 base wall damage per second. Physical hits deal bonus damage against enemies at half health or lower.</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Not rated</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Unrated</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr"/>
+      <c r="H48" s="4" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G45" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
+    <dataValidation sqref="G2:G48" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Use a rating from 1 to 5" error="1 means always skip; 5 means usually take." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="I2:I45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Keep,Rework,Remove,Test first"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Tighten dot drops, scout routes and fresh bomb counters; fix specialist detours
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.126</t>
+          <t>Alpha 0.1.128</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>PROTOTYPE: defeated non-boss monsters have a 10% chance to drop numbered dots: 1, 2, 3 and onward, with no cap or expiry, even across waves. Start at 1, trace at least three numbers in order, then return to 1 in one stroke. Tracing is free. Closing clears the entire batch, including unused dots; the next drop is 1. No combat reward yet. The page shows drops and your biggest loop.</t>
+          <t>PROTOTYPE: defeated non-boss monsters have a 5% chance to drop numbered dots: 1, 2, 3 and onward, with no cap within the wave. Dots clear and numbering restarts at 1 when the wave ends. Start at 1, trace at least three numbers in order, then return to 1 in one stroke. Tracing is free. Closing clears the entire batch, including unused dots; the next drop is 1. No combat reward yet. The page shows drops and your biggest loop.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>PROTOTYPE: defeated non-boss monsters have a 10% chance to drop numbered dots: 1, 2, 3 and onward, with no cap or expiry, even across waves. Start at 1, trace at least three numbers in order, then return to 1 in one stroke. Tracing is free. Closing clears the entire batch, including unused dots; the next drop is 1. No combat reward yet. The page shows drops and your biggest loop.</t>
+          <t>PROTOTYPE: defeated non-boss monsters have a 5% chance to drop numbered dots: 1, 2, 3 and onward, with no cap within the wave. Dots clear and numbering restarts at 1 when the wave ends. Start at 1, trace at least three numbers in order, then return to 1 in one stroke. Tracing is free. Closing clears the entire batch, including unused dots; the next drop is 1. No combat reward yet. The page shows drops and your biggest loop.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Moderate ink and sustain stacking, make tunnels single-use threats, animate Chompzilla
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.128</t>
+          <t>Alpha 0.1.130</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Lines cost 12% less ink.</t>
+          <t>Lines cost 10% less ink per level.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Each level multiplies ink cost by 0.88; a paid stroke still costs at least 6 ink.</t>
+          <t>Each level multiplies ink cost by 0.9; a paid stroke still costs at least 6 ink.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
+          <t>Every kill repairs walls by up to 2.5 HP each, sharing a 10 wall HP/s budget.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Shared repair-on-kill budget: 12 wall HP/s across all walls.</t>
+          <t>Shared repair-on-kill budget: 10 wall HP/s across all walls.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
+          <t>28% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Repeat level n multiplies regeneration by 1 + 0.35 / (1 + 0.5 × (n−1)).</t>
+          <t>Repeat level n multiplies regeneration by 1 + 0.28 / (1 + 0.6 × (n−1)).</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1747,7 +1747,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>Heal 2 HP per kill, sharing the 4.5 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s.</t>
+          <t>Shared combat-healing budget: 4.5 HP/s.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -2678,7 +2678,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 4.5 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Shared combat-healing budget: 6 HP/s; no healing at full health.</t>
+          <t>Shared combat-healing budget: 4.5 HP/s; no healing at full health.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>About 1 second of local active eraser rubbing tears a hole. Each wave starts with fresh paper; wear and holes reset, stay clear of the fort and form shortcuts only to exits at least 45px closer to Stevie. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; paper balls still hit. Rub near the moving bump for 2 seconds to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
+          <t>About 1 second of local active eraser rubbing tears a hole. Each chapter starts with fresh paper; wear and holes persist between waves, stay clear of the fort and lead toward Stevie under the page, stopping at the first subsequent opening crossed. Monsters reaching the fort underneath warn before one armored contact hit and leave without kill rewards. Each monster can enter only once. One 30% entry decision per hole encounter, with no approach-alignment requirement. Bosses never enter. Underground monsters ignore surface effects and damage; paper balls still hit. Rub near the moving bump for 1 second to force a warned emergence and 1.2-second daze. Bosses and airborne boss helpers stay above the page.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Lines cost 12% less ink.</t>
+          <t>Lines cost 10% less ink per level.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Every kill repairs walls by up to 3 HP each, sharing a 12 wall HP/s budget.</t>
+          <t>Every kill repairs walls by up to 2.5 HP each, sharing a 10 wall HP/s budget.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>35% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
+          <t>28% faster ink regeneration on the first pick; smaller multipliers on repeats.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -5744,7 +5744,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Heal 2 HP per kill, sharing the 6 HP/s combat healing budget.</t>
+          <t>Heal 2 HP per kill, sharing the 4.5 HP/s combat healing budget.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 6 HP/s healing budget.</t>
+          <t>Deals life-drain damage on contact; heals up to 1.4 HP/s at rank one, plus 0.375 HP/s per additional rank, from actual damage dealt. Shares the 4.5 HP/s healing budget.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Make Follow the Underline reach distant targets and preserve line rides
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.130</t>
+          <t>Alpha 0.1.131</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Paper balls ride your lines, then launch from the far end with extra range.</t>
+          <t>Paper balls board lines they cross, ride toward the target, then launch from the far end with +100px target range (+30px per extra copy, up to +200px). With no enemy in normal range, Stevie can aim at an open line endpoint within throwing range to reach enemies near its far end. Long rides last until the end; a broken line releases and retargets the ball.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add chapter report cards, build contributions and Gravity Trap whirlpools
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.131</t>
+          <t>Alpha 0.1.132</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Closed loops pull nearby enemies toward their perimeter.</t>
+          <t>Closed loops pull ordinary monsters through their own ink toward a notebook whirlpool. Each monster gets one 15% swallow roll when it reaches a center. Successful gulps share a 1.8-second cooldown; a failed roll briefly dazes it and ends its center pull. Bosses, shields, underground and airborne monsters resist. Other walls and the fort remain solid.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move Discoveries beside monster notes and compact its browser; shorten Blast strokes
</commit_message>
<xml_diff>
--- a/docs/SaveStevie-Upgrade-Reference.xlsx
+++ b/docs/SaveStevie-Upgrade-Reference.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Alpha 0.1.132</t>
+          <t>Alpha 0.1.133</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Walls at least 50px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
+          <t>Walls at least 30px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Walls at least 50px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
+          <t>Walls at least 30px long arm after 0.5s, then explode when destroyed and damage nearby enemies.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">

</xml_diff>